<commit_message>
Limit update provided by Lokesh
</commit_message>
<xml_diff>
--- a/VT LTT Project/Data/Project Database Files/eDCU/48V HighCurrent/Configuration Files/Limit Files/6Head/FE_FF_Frame_Limit_eDCU_Thermal_Endurance_v6.xlsx
+++ b/VT LTT Project/Data/Project Database Files/eDCU/48V HighCurrent/Configuration Files/Limit Files/6Head/FE_FF_Frame_Limit_eDCU_Thermal_Endurance_v6.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eDCU LTT\VT LTT Project\Data\Project Database Files\eDCU\48V HighCurrent\Configuration Files\Limit Files\6Head\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{930DAAD5-B3F6-41D7-91EF-48B92547B1E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE896986-C983-4119-8432-9D7CC86B5B5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{49D2488A-EB0E-4C68-8F67-50F12E4C4F72}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{49D2488A-EB0E-4C68-8F67-50F12E4C4F72}"/>
   </bookViews>
   <sheets>
     <sheet name="Change List" sheetId="5" r:id="rId1"/>
@@ -2640,6 +2640,9 @@
     <xf numFmtId="165" fontId="21" fillId="45" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="46" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="25" fillId="40" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2677,9 +2680,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="42" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="46" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -3871,12 +3871,12 @@
       </c>
       <c r="Z2" s="14"/>
       <c r="AA2" s="14"/>
-      <c r="AB2" s="117">
+      <c r="AB2" s="104">
         <v>160</v>
       </c>
       <c r="AC2" s="14"/>
       <c r="AD2" s="14"/>
-      <c r="AE2" s="117">
+      <c r="AE2" s="104">
         <v>160</v>
       </c>
       <c r="AF2" s="14"/>
@@ -3972,12 +3972,12 @@
       </c>
       <c r="Z3" s="14"/>
       <c r="AA3" s="14"/>
-      <c r="AB3" s="117">
+      <c r="AB3" s="104">
         <v>160</v>
       </c>
       <c r="AC3" s="14"/>
       <c r="AD3" s="14"/>
-      <c r="AE3" s="117">
+      <c r="AE3" s="104">
         <v>160</v>
       </c>
       <c r="AF3" s="14"/>
@@ -4073,12 +4073,12 @@
       </c>
       <c r="Z4" s="14"/>
       <c r="AA4" s="14"/>
-      <c r="AB4" s="117">
+      <c r="AB4" s="104">
         <v>0</v>
       </c>
       <c r="AC4" s="14"/>
       <c r="AD4" s="14"/>
-      <c r="AE4" s="117">
+      <c r="AE4" s="104">
         <v>0</v>
       </c>
       <c r="AF4" s="14"/>
@@ -4174,12 +4174,12 @@
       </c>
       <c r="Z5" s="14"/>
       <c r="AA5" s="14"/>
-      <c r="AB5" s="117">
+      <c r="AB5" s="104">
         <v>0</v>
       </c>
       <c r="AC5" s="14"/>
       <c r="AD5" s="14"/>
-      <c r="AE5" s="117">
+      <c r="AE5" s="104">
         <v>0</v>
       </c>
       <c r="AF5" s="14"/>
@@ -4275,12 +4275,12 @@
       </c>
       <c r="Z6" s="14"/>
       <c r="AA6" s="14"/>
-      <c r="AB6" s="117">
+      <c r="AB6" s="104">
         <v>0</v>
       </c>
       <c r="AC6" s="14"/>
       <c r="AD6" s="14"/>
-      <c r="AE6" s="117">
+      <c r="AE6" s="104">
         <v>0</v>
       </c>
       <c r="AF6" s="14"/>
@@ -4376,12 +4376,12 @@
       </c>
       <c r="Z7" s="14"/>
       <c r="AA7" s="14"/>
-      <c r="AB7" s="117">
+      <c r="AB7" s="104">
         <v>0</v>
       </c>
       <c r="AC7" s="14"/>
       <c r="AD7" s="14"/>
-      <c r="AE7" s="117">
+      <c r="AE7" s="104">
         <v>0</v>
       </c>
       <c r="AF7" s="14"/>
@@ -4477,12 +4477,12 @@
       </c>
       <c r="Z8" s="14"/>
       <c r="AA8" s="14"/>
-      <c r="AB8" s="117">
+      <c r="AB8" s="104">
         <v>0</v>
       </c>
       <c r="AC8" s="14"/>
       <c r="AD8" s="14"/>
-      <c r="AE8" s="117">
+      <c r="AE8" s="104">
         <v>0</v>
       </c>
       <c r="AF8" s="14"/>
@@ -4578,12 +4578,12 @@
       </c>
       <c r="Z9" s="14"/>
       <c r="AA9" s="14"/>
-      <c r="AB9" s="117">
+      <c r="AB9" s="104">
         <v>0</v>
       </c>
       <c r="AC9" s="14"/>
       <c r="AD9" s="14"/>
-      <c r="AE9" s="117">
+      <c r="AE9" s="104">
         <v>0</v>
       </c>
       <c r="AF9" s="14"/>
@@ -4679,12 +4679,12 @@
       </c>
       <c r="Z10" s="14"/>
       <c r="AA10" s="14"/>
-      <c r="AB10" s="117">
+      <c r="AB10" s="104">
         <v>0</v>
       </c>
       <c r="AC10" s="14"/>
       <c r="AD10" s="14"/>
-      <c r="AE10" s="117">
+      <c r="AE10" s="104">
         <v>0</v>
       </c>
       <c r="AF10" s="14"/>
@@ -4780,12 +4780,12 @@
       </c>
       <c r="Z11" s="14"/>
       <c r="AA11" s="14"/>
-      <c r="AB11" s="117">
+      <c r="AB11" s="104">
         <v>0</v>
       </c>
       <c r="AC11" s="14"/>
       <c r="AD11" s="14"/>
-      <c r="AE11" s="117">
+      <c r="AE11" s="104">
         <v>0</v>
       </c>
       <c r="AF11" s="14"/>
@@ -4881,12 +4881,12 @@
       </c>
       <c r="Z12" s="14"/>
       <c r="AA12" s="14"/>
-      <c r="AB12" s="117">
+      <c r="AB12" s="104">
         <v>0</v>
       </c>
       <c r="AC12" s="14"/>
       <c r="AD12" s="14"/>
-      <c r="AE12" s="117">
+      <c r="AE12" s="104">
         <v>0</v>
       </c>
       <c r="AF12" s="14"/>
@@ -4982,12 +4982,12 @@
       </c>
       <c r="Z13" s="14"/>
       <c r="AA13" s="14"/>
-      <c r="AB13" s="117">
+      <c r="AB13" s="104">
         <v>0</v>
       </c>
       <c r="AC13" s="14"/>
       <c r="AD13" s="14"/>
-      <c r="AE13" s="117">
+      <c r="AE13" s="104">
         <v>0</v>
       </c>
       <c r="AF13" s="14"/>
@@ -5083,12 +5083,12 @@
       </c>
       <c r="Z14" s="14"/>
       <c r="AA14" s="14"/>
-      <c r="AB14" s="117">
+      <c r="AB14" s="104">
         <v>160</v>
       </c>
       <c r="AC14" s="14"/>
       <c r="AD14" s="14"/>
-      <c r="AE14" s="117">
+      <c r="AE14" s="104">
         <v>160</v>
       </c>
       <c r="AF14" s="14"/>
@@ -5226,27 +5226,27 @@
         <f>($Y$15*5/Misc!$L$18)+0.1</f>
         <v>2.4690000000000003</v>
       </c>
-      <c r="AB15" s="117">
+      <c r="AB15" s="104">
         <v>2.3690000000000002</v>
       </c>
       <c r="AC15" s="14">
-        <f>($AB$15*5/Misc!$L$19)-0.1</f>
-        <v>2.2690000000000001</v>
+        <f>($AB$15*5/Misc!$L$19)-0.1-0.1</f>
+        <v>2.169</v>
       </c>
       <c r="AD15" s="14">
-        <f>($AB$15*5/Misc!$L$19)+0.1</f>
-        <v>2.4690000000000003</v>
-      </c>
-      <c r="AE15" s="117">
+        <f>($AB$15*5/Misc!$L$19)+0.1+0.1</f>
+        <v>2.5690000000000004</v>
+      </c>
+      <c r="AE15" s="104">
         <v>2.3690000000000002</v>
       </c>
       <c r="AF15" s="14">
-        <f>($AE$15*5/Misc!$L$20)-0.1</f>
-        <v>2.2690000000000001</v>
+        <f>($AE$15*5/Misc!$L$20)-0.1-0.1</f>
+        <v>2.169</v>
       </c>
       <c r="AG15" s="14">
-        <f>($AE$15*5/Misc!$L$20)+0.1</f>
-        <v>2.4690000000000003</v>
+        <f>($AE$15*5/Misc!$L$20)+0.1+0.1</f>
+        <v>2.5690000000000004</v>
       </c>
       <c r="AH15" s="15">
         <v>2.3690000000000002</v>
@@ -5429,27 +5429,27 @@
         <f>($Y$16*5/Misc!$L$18)+0.1</f>
         <v>2.649</v>
       </c>
-      <c r="AB16" s="117">
+      <c r="AB16" s="104">
         <v>2.5489999999999999</v>
       </c>
       <c r="AC16" s="14">
-        <f>($AB$16*5/Misc!$L$19)-0.1</f>
-        <v>2.4489999999999998</v>
+        <f>($AB$16*5/Misc!$L$19)-0.1-0.1</f>
+        <v>2.3489999999999998</v>
       </c>
       <c r="AD16" s="14">
-        <f>($AB$16*5/Misc!$L$19)+0.1</f>
-        <v>2.649</v>
-      </c>
-      <c r="AE16" s="117">
+        <f>($AB$16*5/Misc!$L$19)+0.1+0.1</f>
+        <v>2.7490000000000001</v>
+      </c>
+      <c r="AE16" s="104">
         <v>2.5489999999999999</v>
       </c>
       <c r="AF16" s="14">
-        <f>($AE$16*5/Misc!$L$20)-0.1</f>
-        <v>2.4489999999999998</v>
+        <f>($AE$16*5/Misc!$L$20)-0.1-0.1</f>
+        <v>2.3489999999999998</v>
       </c>
       <c r="AG16" s="14">
-        <f>($AE$16*5/Misc!$L$20)+0.1</f>
-        <v>2.649</v>
+        <f>($AE$16*5/Misc!$L$20)+0.1+0.1</f>
+        <v>2.7490000000000001</v>
       </c>
       <c r="AH16" s="15">
         <v>2.5489999999999999</v>
@@ -5574,10 +5574,10 @@
       <c r="Y17" s="15"/>
       <c r="Z17" s="14"/>
       <c r="AA17" s="14"/>
-      <c r="AB17" s="117"/>
+      <c r="AB17" s="104"/>
       <c r="AC17" s="14"/>
       <c r="AD17" s="14"/>
-      <c r="AE17" s="117"/>
+      <c r="AE17" s="104"/>
       <c r="AF17" s="14"/>
       <c r="AG17" s="14"/>
       <c r="AH17" s="15"/>
@@ -5697,7 +5697,7 @@
         <f>($Y$18*5*1.072/Misc!$L$18)+0.015*3.4</f>
         <v>2.7310000000000003</v>
       </c>
-      <c r="AB18" s="117">
+      <c r="AB18" s="104">
         <v>2.5</v>
       </c>
       <c r="AC18" s="14">
@@ -5708,7 +5708,7 @@
         <f>($AB$18*5*1.072/Misc!$L$19)+0.015*3.4</f>
         <v>2.7310000000000003</v>
       </c>
-      <c r="AE18" s="117">
+      <c r="AE18" s="104">
         <v>2.5</v>
       </c>
       <c r="AF18" s="14">
@@ -5900,7 +5900,7 @@
         <f>($Y$19*5*1.072/Misc!$L$18)+0.015*3.4</f>
         <v>2.7310000000000003</v>
       </c>
-      <c r="AB19" s="117">
+      <c r="AB19" s="104">
         <v>2.5</v>
       </c>
       <c r="AC19" s="14">
@@ -5911,7 +5911,7 @@
         <f>($AB$19*5*1.072/Misc!$L$19)+0.015*3.4</f>
         <v>2.7310000000000003</v>
       </c>
-      <c r="AE19" s="117">
+      <c r="AE19" s="104">
         <v>2.5</v>
       </c>
       <c r="AF19" s="14">
@@ -6045,10 +6045,10 @@
       <c r="Y20" s="15"/>
       <c r="Z20" s="14"/>
       <c r="AA20" s="14"/>
-      <c r="AB20" s="117"/>
+      <c r="AB20" s="104"/>
       <c r="AC20" s="14"/>
       <c r="AD20" s="14"/>
-      <c r="AE20" s="117"/>
+      <c r="AE20" s="104"/>
       <c r="AF20" s="14"/>
       <c r="AG20" s="14"/>
       <c r="AH20" s="15"/>
@@ -6168,7 +6168,7 @@
         <f>(Misc!$J$28*15750/(15750+19860+(Misc!$I$6*219453/(Misc!$I$6+219453))))*(5/Misc!$L$18)+0.02</f>
         <v>0.80722454153136702</v>
       </c>
-      <c r="AB21" s="117">
+      <c r="AB21" s="104">
         <v>0.72</v>
       </c>
       <c r="AC21" s="14">
@@ -6179,7 +6179,7 @@
         <f>(Misc!$J$28*15750/(15750+19860+(Misc!$I$6*219453/(Misc!$I$6+219453))))*(5/Misc!$L$19)+0.02</f>
         <v>0.80722454153136702</v>
       </c>
-      <c r="AE21" s="117">
+      <c r="AE21" s="104">
         <v>0.72</v>
       </c>
       <c r="AF21" s="14">
@@ -6371,7 +6371,7 @@
         <f>(Misc!$K$28*15750/(15750+19860+(Misc!$I$6*219453/(Misc!$I$6+219453))))*(5/Misc!$L$18)+0.02</f>
         <v>0.81514430553067652</v>
       </c>
-      <c r="AB22" s="117">
+      <c r="AB22" s="104">
         <v>0.72</v>
       </c>
       <c r="AC22" s="14">
@@ -6382,7 +6382,7 @@
         <f>(Misc!$K$28*15750/(15750+19860+(Misc!$I$6*219453/(Misc!$I$6+219453))))*(5/Misc!$L$19)+0.02</f>
         <v>0.81514430553067652</v>
       </c>
-      <c r="AE22" s="117">
+      <c r="AE22" s="104">
         <v>0.72</v>
       </c>
       <c r="AF22" s="14">
@@ -6516,10 +6516,10 @@
       <c r="Y23" s="15"/>
       <c r="Z23" s="14"/>
       <c r="AA23" s="14"/>
-      <c r="AB23" s="117"/>
+      <c r="AB23" s="104"/>
       <c r="AC23" s="14"/>
       <c r="AD23" s="14"/>
-      <c r="AE23" s="117"/>
+      <c r="AE23" s="104"/>
       <c r="AF23" s="14"/>
       <c r="AG23" s="14"/>
       <c r="AH23" s="15"/>
@@ -6639,27 +6639,27 @@
         <f>($Y$24*5/Misc!$L$18)+0.015</f>
         <v>2.5010000000000003</v>
       </c>
-      <c r="AB24" s="117">
+      <c r="AB24" s="104">
         <v>2.4860000000000002</v>
       </c>
       <c r="AC24" s="14">
-        <f>($AB$24*5/Misc!$L$19)-0.015</f>
-        <v>2.4710000000000001</v>
+        <f>($AB$24*5/Misc!$L$19)-0.015-0.1</f>
+        <v>2.371</v>
       </c>
       <c r="AD24" s="14">
-        <f>($AB$24*5/Misc!$L$19)+0.015</f>
-        <v>2.5010000000000003</v>
-      </c>
-      <c r="AE24" s="117">
+        <f>($AB$24*5/Misc!$L$19)+0.015+0.1</f>
+        <v>2.6010000000000004</v>
+      </c>
+      <c r="AE24" s="104">
         <v>2.4860000000000002</v>
       </c>
       <c r="AF24" s="14">
-        <f>($AE$24*5/Misc!$L$20)-0.015</f>
-        <v>2.4710000000000001</v>
+        <f>($AE$24*5/Misc!$L$20)-0.015-0.1</f>
+        <v>2.371</v>
       </c>
       <c r="AG24" s="14">
-        <f>($AE$24*5/Misc!$L$20)+0.015</f>
-        <v>2.5010000000000003</v>
+        <f>($AE$24*5/Misc!$L$20)+0.015+0.1</f>
+        <v>2.6010000000000004</v>
       </c>
       <c r="AH24" s="15">
         <v>2.4860000000000002</v>
@@ -6842,27 +6842,27 @@
         <f>($Y$25*5/Misc!$L$18)+0.015</f>
         <v>2.5060000000000002</v>
       </c>
-      <c r="AB25" s="117">
+      <c r="AB25" s="104">
         <v>2.4910000000000001</v>
       </c>
       <c r="AC25" s="14">
-        <f>($AB$25*5/Misc!$L$19)-0.015</f>
-        <v>2.476</v>
+        <f>($AB$25*5/Misc!$L$19)-0.015-0.1</f>
+        <v>2.3759999999999999</v>
       </c>
       <c r="AD25" s="14">
-        <f>($AB$25*5/Misc!$L$19)+0.015</f>
-        <v>2.5060000000000002</v>
-      </c>
-      <c r="AE25" s="117">
+        <f>($AB$25*5/Misc!$L$19)+0.015+0.1</f>
+        <v>2.6060000000000003</v>
+      </c>
+      <c r="AE25" s="104">
         <v>2.4910000000000001</v>
       </c>
       <c r="AF25" s="14">
-        <f>($AE$25*5/Misc!$L$20)-0.015</f>
-        <v>2.476</v>
+        <f>($AE$25*5/Misc!$L$20)-0.015-0.1</f>
+        <v>2.3759999999999999</v>
       </c>
       <c r="AG25" s="14">
-        <f>($AE$25*5/Misc!$L$20)+0.015</f>
-        <v>2.5060000000000002</v>
+        <f>($AE$25*5/Misc!$L$20)+0.015+0.1</f>
+        <v>2.6060000000000003</v>
       </c>
       <c r="AH25" s="15">
         <v>2.4910000000000001</v>
@@ -6987,10 +6987,10 @@
       <c r="Y26" s="15"/>
       <c r="Z26" s="14"/>
       <c r="AA26" s="14"/>
-      <c r="AB26" s="117"/>
+      <c r="AB26" s="104"/>
       <c r="AC26" s="14"/>
       <c r="AD26" s="14"/>
-      <c r="AE26" s="117"/>
+      <c r="AE26" s="104"/>
       <c r="AF26" s="14"/>
       <c r="AG26" s="14"/>
       <c r="AH26" s="15"/>
@@ -7110,7 +7110,7 @@
         <f>(Misc!$H$28)*(5*1.008/Misc!$L$18)+0.02*1.1</f>
         <v>5.0317600000000002</v>
       </c>
-      <c r="AB27" s="117">
+      <c r="AB27" s="104">
         <v>4.9950000000000001</v>
       </c>
       <c r="AC27" s="14">
@@ -7121,7 +7121,7 @@
         <f>(Misc!$H$28)*(5*1.008/Misc!$L$19)+0.02*1.1</f>
         <v>5.0317600000000002</v>
       </c>
-      <c r="AE27" s="117">
+      <c r="AE27" s="104">
         <v>4.9950000000000001</v>
       </c>
       <c r="AF27" s="14">
@@ -7301,7 +7301,7 @@
         <f>(Misc!$I$28)*(5*1.008/Misc!$L$18)+0.02*1.1</f>
         <v>5.08216</v>
       </c>
-      <c r="AB28" s="117">
+      <c r="AB28" s="104">
         <v>5</v>
       </c>
       <c r="AC28" s="14">
@@ -7312,7 +7312,7 @@
         <f>(Misc!$I$28)*(5*1.008/Misc!$L$19)+0.02*1.1</f>
         <v>5.08216</v>
       </c>
-      <c r="AE28" s="117">
+      <c r="AE28" s="104">
         <v>5</v>
       </c>
       <c r="AF28" s="14">
@@ -7434,10 +7434,10 @@
       <c r="Y29" s="15"/>
       <c r="Z29" s="14"/>
       <c r="AA29" s="14"/>
-      <c r="AB29" s="117"/>
+      <c r="AB29" s="104"/>
       <c r="AC29" s="14"/>
       <c r="AD29" s="14"/>
-      <c r="AE29" s="117"/>
+      <c r="AE29" s="104"/>
       <c r="AF29" s="14"/>
       <c r="AG29" s="14"/>
       <c r="AH29" s="15"/>
@@ -7557,7 +7557,7 @@
         <f>($Y$30*5*1.072/Misc!$L$18)+0.02*3.4</f>
         <v>2.7480000000000002</v>
       </c>
-      <c r="AB30" s="117">
+      <c r="AB30" s="104">
         <v>2.5</v>
       </c>
       <c r="AC30" s="14">
@@ -7568,7 +7568,7 @@
         <f>($AB$30*5*1.072/Misc!$L$19)+0.02*3.4</f>
         <v>2.7480000000000002</v>
       </c>
-      <c r="AE30" s="117">
+      <c r="AE30" s="104">
         <v>2.5</v>
       </c>
       <c r="AF30" s="14">
@@ -7760,7 +7760,7 @@
         <f>($Y$31*5*1.072/Misc!$L$18)+0.02*3.4</f>
         <v>2.7480000000000002</v>
       </c>
-      <c r="AB31" s="117">
+      <c r="AB31" s="104">
         <v>2.5</v>
       </c>
       <c r="AC31" s="14">
@@ -7771,7 +7771,7 @@
         <f>($AB$31*5*1.072/Misc!$L$19)+0.02*3.4</f>
         <v>2.7480000000000002</v>
       </c>
-      <c r="AE31" s="117">
+      <c r="AE31" s="104">
         <v>2.5</v>
       </c>
       <c r="AF31" s="14">
@@ -7905,10 +7905,10 @@
       <c r="Y32" s="15"/>
       <c r="Z32" s="14"/>
       <c r="AA32" s="14"/>
-      <c r="AB32" s="117"/>
+      <c r="AB32" s="104"/>
       <c r="AC32" s="14"/>
       <c r="AD32" s="14"/>
-      <c r="AE32" s="117"/>
+      <c r="AE32" s="104"/>
       <c r="AF32" s="14"/>
       <c r="AG32" s="14"/>
       <c r="AH32" s="15"/>
@@ -8028,7 +8028,7 @@
         <f>($Y$33*5*1.072/Misc!$L$18)+0.02*3.4</f>
         <v>2.7480000000000002</v>
       </c>
-      <c r="AB33" s="117">
+      <c r="AB33" s="104">
         <v>2.5</v>
       </c>
       <c r="AC33" s="14">
@@ -8039,7 +8039,7 @@
         <f>($AB$33*5*1.072/Misc!$L$19)+0.02*3.4</f>
         <v>2.7480000000000002</v>
       </c>
-      <c r="AE33" s="117">
+      <c r="AE33" s="104">
         <v>2.5</v>
       </c>
       <c r="AF33" s="14">
@@ -8231,7 +8231,7 @@
         <f>($Y$34*5*1.072/Misc!$L$18)+0.02*3.4</f>
         <v>2.7480000000000002</v>
       </c>
-      <c r="AB34" s="117">
+      <c r="AB34" s="104">
         <v>2.5</v>
       </c>
       <c r="AC34" s="14">
@@ -8242,7 +8242,7 @@
         <f>($AB$34*5*1.072/Misc!$L$19)+0.02*3.4</f>
         <v>2.7480000000000002</v>
       </c>
-      <c r="AE34" s="117">
+      <c r="AE34" s="104">
         <v>2.5</v>
       </c>
       <c r="AF34" s="14">
@@ -8376,10 +8376,10 @@
       <c r="Y35" s="15"/>
       <c r="Z35" s="14"/>
       <c r="AA35" s="14"/>
-      <c r="AB35" s="117"/>
+      <c r="AB35" s="104"/>
       <c r="AC35" s="14"/>
       <c r="AD35" s="14"/>
-      <c r="AE35" s="117"/>
+      <c r="AE35" s="104"/>
       <c r="AF35" s="14"/>
       <c r="AG35" s="14"/>
       <c r="AH35" s="15"/>
@@ -8485,7 +8485,7 @@
         <f>Misc!$K$18*1.05</f>
         <v>124.95</v>
       </c>
-      <c r="AB36" s="117"/>
+      <c r="AB36" s="104"/>
       <c r="AC36" s="14">
         <f>Misc!$J$19*1.05</f>
         <v>-21</v>
@@ -8494,7 +8494,7 @@
         <f>Misc!$K$19*1.05</f>
         <v>124.95</v>
       </c>
-      <c r="AE36" s="117"/>
+      <c r="AE36" s="104"/>
       <c r="AF36" s="14">
         <f>Misc!$J$20*1.05</f>
         <v>-21</v>
@@ -8653,7 +8653,7 @@
         <f>Misc!$K$18*1.05</f>
         <v>124.95</v>
       </c>
-      <c r="AB37" s="117"/>
+      <c r="AB37" s="104"/>
       <c r="AC37" s="14">
         <f>Misc!$J$19*1.05</f>
         <v>-21</v>
@@ -8662,7 +8662,7 @@
         <f>Misc!$K$19*1.05</f>
         <v>124.95</v>
       </c>
-      <c r="AE37" s="117"/>
+      <c r="AE37" s="104"/>
       <c r="AF37" s="14">
         <f>Misc!$J$20*1.05</f>
         <v>-21</v>
@@ -8777,10 +8777,10 @@
       <c r="Y38" s="15"/>
       <c r="Z38" s="14"/>
       <c r="AA38" s="14"/>
-      <c r="AB38" s="117"/>
+      <c r="AB38" s="104"/>
       <c r="AC38" s="14"/>
       <c r="AD38" s="14"/>
-      <c r="AE38" s="117"/>
+      <c r="AE38" s="104"/>
       <c r="AF38" s="14"/>
       <c r="AG38" s="14"/>
       <c r="AH38" s="15"/>
@@ -8900,7 +8900,7 @@
         <f>($Y$39*5*1.072/Misc!$L$18)+0.02*3.4</f>
         <v>2.7480000000000002</v>
       </c>
-      <c r="AB39" s="117">
+      <c r="AB39" s="104">
         <v>2.5</v>
       </c>
       <c r="AC39" s="14">
@@ -8911,7 +8911,7 @@
         <f>($AB$39*5*1.072/Misc!$L$19)+0.02*3.4</f>
         <v>2.7480000000000002</v>
       </c>
-      <c r="AE39" s="117">
+      <c r="AE39" s="104">
         <v>2.5</v>
       </c>
       <c r="AF39" s="14">
@@ -9103,7 +9103,7 @@
         <f>($Y$40*5*1.072/Misc!$L$18)+0.02*3.4</f>
         <v>2.7480000000000002</v>
       </c>
-      <c r="AB40" s="117">
+      <c r="AB40" s="104">
         <v>2.5</v>
       </c>
       <c r="AC40" s="14">
@@ -9114,7 +9114,7 @@
         <f>($AB$40*5*1.072/Misc!$L$19)+0.02*3.4</f>
         <v>2.7480000000000002</v>
       </c>
-      <c r="AE40" s="117">
+      <c r="AE40" s="104">
         <v>2.5</v>
       </c>
       <c r="AF40" s="14">
@@ -9248,10 +9248,10 @@
       <c r="Y41" s="15"/>
       <c r="Z41" s="14"/>
       <c r="AA41" s="14"/>
-      <c r="AB41" s="117"/>
+      <c r="AB41" s="104"/>
       <c r="AC41" s="14"/>
       <c r="AD41" s="14"/>
-      <c r="AE41" s="117"/>
+      <c r="AE41" s="104"/>
       <c r="AF41" s="14"/>
       <c r="AG41" s="14"/>
       <c r="AH41" s="15"/>
@@ -9371,7 +9371,7 @@
         <f>($Y$42*5*1.064/Misc!$L$18)+0.02*2.8</f>
         <v>2.7160000000000002</v>
       </c>
-      <c r="AB42" s="117">
+      <c r="AB42" s="104">
         <v>2.5</v>
       </c>
       <c r="AC42" s="14">
@@ -9382,7 +9382,7 @@
         <f>($AB$42*5*1.064/Misc!$L$19)+0.02*2.8</f>
         <v>2.7160000000000002</v>
       </c>
-      <c r="AE42" s="117">
+      <c r="AE42" s="104">
         <v>2.5</v>
       </c>
       <c r="AF42" s="14">
@@ -9574,7 +9574,7 @@
         <f>($Y$43*5*1.064/Misc!$L$18)+0.02*2.8</f>
         <v>2.7160000000000002</v>
       </c>
-      <c r="AB43" s="117">
+      <c r="AB43" s="104">
         <v>2.5</v>
       </c>
       <c r="AC43" s="14">
@@ -9585,7 +9585,7 @@
         <f>($AB$43*5*1.064/Misc!$L$19)+0.02*2.8</f>
         <v>2.7160000000000002</v>
       </c>
-      <c r="AE43" s="117">
+      <c r="AE43" s="104">
         <v>2.5</v>
       </c>
       <c r="AF43" s="14">
@@ -9719,10 +9719,10 @@
       <c r="Y44" s="15"/>
       <c r="Z44" s="14"/>
       <c r="AA44" s="14"/>
-      <c r="AB44" s="117"/>
+      <c r="AB44" s="104"/>
       <c r="AC44" s="14"/>
       <c r="AD44" s="14"/>
-      <c r="AE44" s="117"/>
+      <c r="AE44" s="104"/>
       <c r="AF44" s="14"/>
       <c r="AG44" s="14"/>
       <c r="AH44" s="15"/>
@@ -9842,7 +9842,7 @@
         <f>($Y$45*5*1.072/Misc!$L$18)+0.02*3.4</f>
         <v>2.7480000000000002</v>
       </c>
-      <c r="AB45" s="117">
+      <c r="AB45" s="104">
         <v>2.5</v>
       </c>
       <c r="AC45" s="14">
@@ -9853,7 +9853,7 @@
         <f>($AB$45*5*1.072/Misc!$L$19)+0.02*3.4</f>
         <v>2.7480000000000002</v>
       </c>
-      <c r="AE45" s="117">
+      <c r="AE45" s="104">
         <v>2.5</v>
       </c>
       <c r="AF45" s="14">
@@ -10045,7 +10045,7 @@
         <f>($Y$46*5*1.072/Misc!$L$18)+0.02*3.4</f>
         <v>2.7480000000000002</v>
       </c>
-      <c r="AB46" s="117">
+      <c r="AB46" s="104">
         <v>2.5</v>
       </c>
       <c r="AC46" s="14">
@@ -10056,7 +10056,7 @@
         <f>($AB$46*5*1.072/Misc!$L$19)+0.02*3.4</f>
         <v>2.7480000000000002</v>
       </c>
-      <c r="AE46" s="117">
+      <c r="AE46" s="104">
         <v>2.5</v>
       </c>
       <c r="AF46" s="14">
@@ -10190,10 +10190,10 @@
       <c r="Y47" s="15"/>
       <c r="Z47" s="14"/>
       <c r="AA47" s="14"/>
-      <c r="AB47" s="117"/>
+      <c r="AB47" s="104"/>
       <c r="AC47" s="14"/>
       <c r="AD47" s="14"/>
-      <c r="AE47" s="117"/>
+      <c r="AE47" s="104"/>
       <c r="AF47" s="14"/>
       <c r="AG47" s="14"/>
       <c r="AH47" s="15"/>
@@ -10313,7 +10313,7 @@
         <f>($Y$48*5*1.072/Misc!$L$18)+0.02*3.4</f>
         <v>2.7480000000000002</v>
       </c>
-      <c r="AB48" s="117">
+      <c r="AB48" s="104">
         <v>2.5</v>
       </c>
       <c r="AC48" s="14">
@@ -10324,7 +10324,7 @@
         <f>($AB$48*5*1.072/Misc!$L$19)+0.02*3.4</f>
         <v>2.7480000000000002</v>
       </c>
-      <c r="AE48" s="117">
+      <c r="AE48" s="104">
         <v>2.5</v>
       </c>
       <c r="AF48" s="14">
@@ -10516,7 +10516,7 @@
         <f>($Y$49*5*1.072/Misc!$L$18)+0.02*3.4</f>
         <v>2.7480000000000002</v>
       </c>
-      <c r="AB49" s="117">
+      <c r="AB49" s="104">
         <v>2.5</v>
       </c>
       <c r="AC49" s="14">
@@ -10527,7 +10527,7 @@
         <f>($AB$49*5*1.072/Misc!$L$19)+0.02*3.4</f>
         <v>2.7480000000000002</v>
       </c>
-      <c r="AE49" s="117">
+      <c r="AE49" s="104">
         <v>2.5</v>
       </c>
       <c r="AF49" s="14">
@@ -10661,10 +10661,10 @@
       <c r="Y50" s="15"/>
       <c r="Z50" s="14"/>
       <c r="AA50" s="14"/>
-      <c r="AB50" s="117"/>
+      <c r="AB50" s="104"/>
       <c r="AC50" s="14"/>
       <c r="AD50" s="14"/>
-      <c r="AE50" s="117"/>
+      <c r="AE50" s="104"/>
       <c r="AF50" s="14"/>
       <c r="AG50" s="14"/>
       <c r="AH50" s="15"/>
@@ -10784,7 +10784,7 @@
         <f>($Y$51*5*1.064/Misc!$L$18)+0.02*2.8</f>
         <v>2.7160000000000002</v>
       </c>
-      <c r="AB51" s="117">
+      <c r="AB51" s="104">
         <v>2.5</v>
       </c>
       <c r="AC51" s="14">
@@ -10795,7 +10795,7 @@
         <f>($AB$51*5*1.064/Misc!$L$19)+0.02*2.8</f>
         <v>2.7160000000000002</v>
       </c>
-      <c r="AE51" s="117">
+      <c r="AE51" s="104">
         <v>2.5</v>
       </c>
       <c r="AF51" s="14">
@@ -10987,7 +10987,7 @@
         <f>($Y$52*5*1.064/Misc!$L$18)+0.02*2.8</f>
         <v>2.7160000000000002</v>
       </c>
-      <c r="AB52" s="117">
+      <c r="AB52" s="104">
         <v>2.5</v>
       </c>
       <c r="AC52" s="14">
@@ -10998,7 +10998,7 @@
         <f>($AB$52*5*1.064/Misc!$L$19)+0.02*2.8</f>
         <v>2.7160000000000002</v>
       </c>
-      <c r="AE52" s="117">
+      <c r="AE52" s="104">
         <v>2.5</v>
       </c>
       <c r="AF52" s="14">
@@ -11132,10 +11132,10 @@
       <c r="Y53" s="15"/>
       <c r="Z53" s="14"/>
       <c r="AA53" s="14"/>
-      <c r="AB53" s="117"/>
+      <c r="AB53" s="104"/>
       <c r="AC53" s="14"/>
       <c r="AD53" s="14"/>
-      <c r="AE53" s="117"/>
+      <c r="AE53" s="104"/>
       <c r="AF53" s="14"/>
       <c r="AG53" s="14"/>
       <c r="AH53" s="15"/>
@@ -11255,27 +11255,27 @@
         <f>($Y$54*5/Misc!$L$18)+0.1</f>
         <v>2.468</v>
       </c>
-      <c r="AB54" s="117">
+      <c r="AB54" s="104">
         <v>2.3679999999999999</v>
       </c>
       <c r="AC54" s="14">
-        <f>($AB$54*5/Misc!$L$19)-0.1</f>
-        <v>2.2679999999999998</v>
+        <f>($AB$54*5/Misc!$L$19)-0.1-0.1</f>
+        <v>2.1679999999999997</v>
       </c>
       <c r="AD54" s="14">
-        <f>($AB$54*5/Misc!$L$19)+0.1</f>
-        <v>2.468</v>
-      </c>
-      <c r="AE54" s="117">
+        <f>($AB$54*5/Misc!$L$19)+0.1+0.1</f>
+        <v>2.5680000000000001</v>
+      </c>
+      <c r="AE54" s="104">
         <v>2.3679999999999999</v>
       </c>
       <c r="AF54" s="14">
-        <f>($AE$54*5/Misc!$L$20)-0.1</f>
-        <v>2.2679999999999998</v>
+        <f>($AE$54*5/Misc!$L$20)-0.1-0.1</f>
+        <v>2.1679999999999997</v>
       </c>
       <c r="AG54" s="14">
-        <f>($AE$54*5/Misc!$L$20)+0.1</f>
-        <v>2.468</v>
+        <f>($AE$54*5/Misc!$L$20)+0.1+0.1</f>
+        <v>2.5680000000000001</v>
       </c>
       <c r="AH54" s="15">
         <v>2.3679999999999999</v>
@@ -11458,27 +11458,27 @@
         <f>($Y$55*5/Misc!$L$18)+0.1</f>
         <v>2.633</v>
       </c>
-      <c r="AB55" s="117">
+      <c r="AB55" s="104">
         <v>2.5329999999999999</v>
       </c>
       <c r="AC55" s="14">
-        <f>($AB$55*5/Misc!$L$19)-0.1</f>
-        <v>2.4329999999999998</v>
+        <f>($AB$55*5/Misc!$L$19)-0.1-0.1</f>
+        <v>2.3329999999999997</v>
       </c>
       <c r="AD55" s="14">
-        <f>($AB$55*5/Misc!$L$19)+0.1</f>
-        <v>2.633</v>
-      </c>
-      <c r="AE55" s="117">
+        <f>($AB$55*5/Misc!$L$19)+0.1+0.1</f>
+        <v>2.7330000000000001</v>
+      </c>
+      <c r="AE55" s="104">
         <v>2.5329999999999999</v>
       </c>
       <c r="AF55" s="14">
-        <f>($AE$55*5/Misc!$L$20)-0.1</f>
-        <v>2.4329999999999998</v>
+        <f>($AE$55*5/Misc!$L$20)-0.1-0.1</f>
+        <v>2.3329999999999997</v>
       </c>
       <c r="AG55" s="14">
-        <f>($AE$55*5/Misc!$L$20)+0.1</f>
-        <v>2.633</v>
+        <f>($AE$55*5/Misc!$L$20)+0.1+0.1</f>
+        <v>2.7330000000000001</v>
       </c>
       <c r="AH55" s="15">
         <v>2.5329999999999999</v>
@@ -11603,10 +11603,10 @@
       <c r="Y56" s="15"/>
       <c r="Z56" s="14"/>
       <c r="AA56" s="14"/>
-      <c r="AB56" s="117"/>
+      <c r="AB56" s="104"/>
       <c r="AC56" s="14"/>
       <c r="AD56" s="14"/>
-      <c r="AE56" s="117"/>
+      <c r="AE56" s="104"/>
       <c r="AF56" s="14"/>
       <c r="AG56" s="14"/>
       <c r="AH56" s="15"/>
@@ -11726,7 +11726,7 @@
         <f>($Y$57*5*1.072/Misc!$L$18)+0.015*3.4</f>
         <v>2.7310000000000003</v>
       </c>
-      <c r="AB57" s="117">
+      <c r="AB57" s="104">
         <v>2.5</v>
       </c>
       <c r="AC57" s="14">
@@ -11737,7 +11737,7 @@
         <f>($AB$57*5*1.072/Misc!$L$19)+0.015*3.4</f>
         <v>2.7310000000000003</v>
       </c>
-      <c r="AE57" s="117">
+      <c r="AE57" s="104">
         <v>2.5</v>
       </c>
       <c r="AF57" s="14">
@@ -11929,7 +11929,7 @@
         <f>($Y$58*5*1.072/Misc!$L$18)+0.015*3.4</f>
         <v>2.7310000000000003</v>
       </c>
-      <c r="AB58" s="117">
+      <c r="AB58" s="104">
         <v>2.5</v>
       </c>
       <c r="AC58" s="14">
@@ -11940,7 +11940,7 @@
         <f>($AB$58*5*1.072/Misc!$L$19)+0.015*3.4</f>
         <v>2.7310000000000003</v>
       </c>
-      <c r="AE58" s="117">
+      <c r="AE58" s="104">
         <v>2.5</v>
       </c>
       <c r="AF58" s="14">
@@ -12074,10 +12074,10 @@
       <c r="Y59" s="15"/>
       <c r="Z59" s="14"/>
       <c r="AA59" s="14"/>
-      <c r="AB59" s="117"/>
+      <c r="AB59" s="104"/>
       <c r="AC59" s="14"/>
       <c r="AD59" s="14"/>
-      <c r="AE59" s="117"/>
+      <c r="AE59" s="104"/>
       <c r="AF59" s="14"/>
       <c r="AG59" s="14"/>
       <c r="AH59" s="15"/>
@@ -12197,7 +12197,7 @@
         <f>((Misc!$J$28*(222547*Misc!$J$6/(222547+Misc!$J$6)+15750)/((222547*Misc!$J$6/(222547+Misc!$J$6)+15750)+19860))*(5/Misc!$L$18))+0.02</f>
         <v>4.0863153688422091</v>
       </c>
-      <c r="AB60" s="117">
+      <c r="AB60" s="104">
         <v>4</v>
       </c>
       <c r="AC60" s="14">
@@ -12208,7 +12208,7 @@
         <f>((Misc!$J$28*(222547*Misc!$J$6/(222547+Misc!$J$6)+15750)/((222547*Misc!$J$6/(222547+Misc!$J$6)+15750)+19860))*(5/Misc!$L$19))+0.02</f>
         <v>4.0863153688422091</v>
       </c>
-      <c r="AE60" s="117">
+      <c r="AE60" s="104">
         <v>4</v>
       </c>
       <c r="AF60" s="14">
@@ -12386,7 +12386,7 @@
         <f>((Misc!$K$28*(222547*Misc!$J$6/(222547+Misc!$J$6)+15750)/((222547*Misc!$J$6/(222547+Misc!$J$6)+15750)+19860))*(5/Misc!$L$18))+0.02</f>
         <v>4.1272239741625532</v>
       </c>
-      <c r="AB61" s="117">
+      <c r="AB61" s="104">
         <v>4</v>
       </c>
       <c r="AC61" s="14">
@@ -12397,7 +12397,7 @@
         <f>((Misc!$K$28*(222547*Misc!$J$6/(222547+Misc!$J$6)+15750)/((222547*Misc!$J$6/(222547+Misc!$J$6)+15750)+19860))*(5/Misc!$L$19))+0.02</f>
         <v>4.1272239741625532</v>
       </c>
-      <c r="AE61" s="117">
+      <c r="AE61" s="104">
         <v>4</v>
       </c>
       <c r="AF61" s="14">
@@ -12517,10 +12517,10 @@
       <c r="Y62" s="15"/>
       <c r="Z62" s="14"/>
       <c r="AA62" s="14"/>
-      <c r="AB62" s="117"/>
+      <c r="AB62" s="104"/>
       <c r="AC62" s="14"/>
       <c r="AD62" s="14"/>
-      <c r="AE62" s="117"/>
+      <c r="AE62" s="104"/>
       <c r="AF62" s="14"/>
       <c r="AG62" s="14"/>
       <c r="AH62" s="15"/>
@@ -12640,27 +12640,27 @@
         <f>($Y$63*5/Misc!$L$18)+0.015</f>
         <v>2.4900000000000002</v>
       </c>
-      <c r="AB63" s="117">
+      <c r="AB63" s="104">
         <v>2.4750000000000001</v>
       </c>
       <c r="AC63" s="14">
-        <f>($AB$63*5/Misc!$L$19)-0.015</f>
-        <v>2.46</v>
+        <f>($AB$63*5/Misc!$L$19)-0.015-0.05</f>
+        <v>2.41</v>
       </c>
       <c r="AD63" s="14">
-        <f>($AB$63*5/Misc!$L$19)+0.015</f>
-        <v>2.4900000000000002</v>
-      </c>
-      <c r="AE63" s="117">
+        <f>($AB$63*5/Misc!$L$19)+0.015+0.05</f>
+        <v>2.54</v>
+      </c>
+      <c r="AE63" s="104">
         <v>2.4750000000000001</v>
       </c>
       <c r="AF63" s="14">
-        <f>($AE$63*5/Misc!$L$20)-0.015</f>
-        <v>2.46</v>
+        <f>($AE$63*5/Misc!$L$20)-0.015-0.05</f>
+        <v>2.41</v>
       </c>
       <c r="AG63" s="14">
-        <f>($AE$63*5/Misc!$L$20)+0.015</f>
-        <v>2.4900000000000002</v>
+        <f>($AE$63*5/Misc!$L$20)+0.015+0.05</f>
+        <v>2.54</v>
       </c>
       <c r="AH63" s="15">
         <v>2.4750000000000001</v>
@@ -12843,27 +12843,27 @@
         <f>($Y$64*5/Misc!$L$18)+0.015</f>
         <v>2.4940000000000002</v>
       </c>
-      <c r="AB64" s="117">
+      <c r="AB64" s="104">
         <v>2.4790000000000001</v>
       </c>
       <c r="AC64" s="14">
-        <f>($AB$64*5/Misc!$L$19)-0.015</f>
-        <v>2.464</v>
+        <f>($AB$64*5/Misc!$L$19)-0.015-0.05</f>
+        <v>2.4140000000000001</v>
       </c>
       <c r="AD64" s="14">
-        <f>($AB$64*5/Misc!$L$19)+0.015</f>
-        <v>2.4940000000000002</v>
-      </c>
-      <c r="AE64" s="117">
+        <f>($AB$64*5/Misc!$L$19)+0.015+0.05</f>
+        <v>2.544</v>
+      </c>
+      <c r="AE64" s="104">
         <v>2.4790000000000001</v>
       </c>
       <c r="AF64" s="14">
-        <f>($AE$64*5/Misc!$L$20)-0.015</f>
-        <v>2.464</v>
+        <f>($AE$64*5/Misc!$L$20)-0.015-0.05</f>
+        <v>2.4140000000000001</v>
       </c>
       <c r="AG64" s="14">
-        <f>($AE$64*5/Misc!$L$20)+0.015</f>
-        <v>2.4940000000000002</v>
+        <f>($AE$64*5/Misc!$L$20)+0.015+0.05</f>
+        <v>2.544</v>
       </c>
       <c r="AH64" s="15">
         <v>2.4790000000000001</v>
@@ -12988,10 +12988,10 @@
       <c r="Y65" s="15"/>
       <c r="Z65" s="14"/>
       <c r="AA65" s="14"/>
-      <c r="AB65" s="117"/>
+      <c r="AB65" s="104"/>
       <c r="AC65" s="14"/>
       <c r="AD65" s="14"/>
-      <c r="AE65" s="117"/>
+      <c r="AE65" s="104"/>
       <c r="AF65" s="14"/>
       <c r="AG65" s="14"/>
       <c r="AH65" s="15"/>
@@ -13111,7 +13111,7 @@
         <f>($Y$66)*(5*1.074/Misc!$L$18)+0.02*4.13</f>
         <v>12.949120000000001</v>
       </c>
-      <c r="AB66" s="117">
+      <c r="AB66" s="104">
         <v>11.98</v>
       </c>
       <c r="AC66" s="14">
@@ -13122,7 +13122,7 @@
         <f>($AB$66)*(5*1.074/Misc!$L$19)+0.02*4.13</f>
         <v>12.949120000000001</v>
       </c>
-      <c r="AE66" s="117">
+      <c r="AE66" s="104">
         <v>11.98</v>
       </c>
       <c r="AF66" s="14">
@@ -13314,7 +13314,7 @@
         <f>($Y$67)*(5*1.074/Misc!$L$18)+0.02*4.13</f>
         <v>12.970600000000001</v>
       </c>
-      <c r="AB67" s="117">
+      <c r="AB67" s="104">
         <v>12</v>
       </c>
       <c r="AC67" s="14">
@@ -13325,7 +13325,7 @@
         <f>($AB$67)*(5*1.074/Misc!$L$19)+0.02*4.13</f>
         <v>12.970600000000001</v>
       </c>
-      <c r="AE67" s="117">
+      <c r="AE67" s="104">
         <v>12</v>
       </c>
       <c r="AF67" s="14">
@@ -13459,10 +13459,10 @@
       <c r="Y68" s="15"/>
       <c r="Z68" s="14"/>
       <c r="AA68" s="14"/>
-      <c r="AB68" s="117"/>
+      <c r="AB68" s="104"/>
       <c r="AC68" s="14"/>
       <c r="AD68" s="14"/>
-      <c r="AE68" s="117"/>
+      <c r="AE68" s="104"/>
       <c r="AF68" s="14"/>
       <c r="AG68" s="14"/>
       <c r="AH68" s="15"/>
@@ -13582,7 +13582,7 @@
         <f>($Y$69*5*1.072/Misc!$L$18)+0.015*3.4</f>
         <v>2.7310000000000003</v>
       </c>
-      <c r="AB69" s="117">
+      <c r="AB69" s="104">
         <v>2.5</v>
       </c>
       <c r="AC69" s="14">
@@ -13593,7 +13593,7 @@
         <f>($AB$69*5*1.072/Misc!$L$19)+0.015*3.4</f>
         <v>2.7310000000000003</v>
       </c>
-      <c r="AE69" s="117">
+      <c r="AE69" s="104">
         <v>2.5</v>
       </c>
       <c r="AF69" s="14">
@@ -13785,7 +13785,7 @@
         <f>($Y$70*5*1.072/Misc!$L$18)+0.015*3.4</f>
         <v>2.7310000000000003</v>
       </c>
-      <c r="AB70" s="117">
+      <c r="AB70" s="104">
         <v>2.5</v>
       </c>
       <c r="AC70" s="14">
@@ -13796,7 +13796,7 @@
         <f>($AB$70*5*1.072/Misc!$L$19)+0.015*3.4</f>
         <v>2.7310000000000003</v>
       </c>
-      <c r="AE70" s="117">
+      <c r="AE70" s="104">
         <v>2.5</v>
       </c>
       <c r="AF70" s="14">
@@ -13930,10 +13930,10 @@
       <c r="Y71" s="15"/>
       <c r="Z71" s="14"/>
       <c r="AA71" s="14"/>
-      <c r="AB71" s="117"/>
+      <c r="AB71" s="104"/>
       <c r="AC71" s="14"/>
       <c r="AD71" s="14"/>
-      <c r="AE71" s="117"/>
+      <c r="AE71" s="104"/>
       <c r="AF71" s="14"/>
       <c r="AG71" s="14"/>
       <c r="AH71" s="15"/>
@@ -14053,7 +14053,7 @@
         <f>($Y$72*5*1.072/Misc!$L$18)+0.015*3.4</f>
         <v>2.7310000000000003</v>
       </c>
-      <c r="AB72" s="117">
+      <c r="AB72" s="104">
         <v>2.5</v>
       </c>
       <c r="AC72" s="14">
@@ -14064,7 +14064,7 @@
         <f>($AB$72*5*1.072/Misc!$L$19)+0.015*3.4</f>
         <v>2.7310000000000003</v>
       </c>
-      <c r="AE72" s="117">
+      <c r="AE72" s="104">
         <v>2.5</v>
       </c>
       <c r="AF72" s="14">
@@ -14256,7 +14256,7 @@
         <f>($Y$73*5*1.072/Misc!$L$18)+0.015*3.4</f>
         <v>2.7310000000000003</v>
       </c>
-      <c r="AB73" s="117">
+      <c r="AB73" s="104">
         <v>2.5</v>
       </c>
       <c r="AC73" s="14">
@@ -14267,7 +14267,7 @@
         <f>($AB$73*5*1.072/Misc!$L$19)+0.015*3.4</f>
         <v>2.7310000000000003</v>
       </c>
-      <c r="AE73" s="117">
+      <c r="AE73" s="104">
         <v>2.5</v>
       </c>
       <c r="AF73" s="14">
@@ -14401,10 +14401,10 @@
       <c r="Y74" s="15"/>
       <c r="Z74" s="14"/>
       <c r="AA74" s="14"/>
-      <c r="AB74" s="117"/>
+      <c r="AB74" s="104"/>
       <c r="AC74" s="14"/>
       <c r="AD74" s="14"/>
-      <c r="AE74" s="117"/>
+      <c r="AE74" s="104"/>
       <c r="AF74" s="14"/>
       <c r="AG74" s="14"/>
       <c r="AH74" s="15"/>
@@ -14524,7 +14524,7 @@
         <f>($Y$75*5*1.072/Misc!$L$18)+0.015*3.4</f>
         <v>2.7310000000000003</v>
       </c>
-      <c r="AB75" s="117">
+      <c r="AB75" s="104">
         <v>2.5</v>
       </c>
       <c r="AC75" s="14">
@@ -14535,7 +14535,7 @@
         <f>($AB$75*5*1.072/Misc!$L$19)+0.015*3.4</f>
         <v>2.7310000000000003</v>
       </c>
-      <c r="AE75" s="117">
+      <c r="AE75" s="104">
         <v>2.5</v>
       </c>
       <c r="AF75" s="14">
@@ -14727,7 +14727,7 @@
         <f>($Y$76*5*1.072/Misc!$L$18)+0.015*3.4</f>
         <v>2.7310000000000003</v>
       </c>
-      <c r="AB76" s="117">
+      <c r="AB76" s="104">
         <v>2.5</v>
       </c>
       <c r="AC76" s="14">
@@ -14738,7 +14738,7 @@
         <f>($AB$76*5*1.072/Misc!$L$19)+0.015*3.4</f>
         <v>2.7310000000000003</v>
       </c>
-      <c r="AE76" s="117">
+      <c r="AE76" s="104">
         <v>2.5</v>
       </c>
       <c r="AF76" s="14">
@@ -14872,10 +14872,10 @@
       <c r="Y77" s="15"/>
       <c r="Z77" s="14"/>
       <c r="AA77" s="14"/>
-      <c r="AB77" s="117"/>
+      <c r="AB77" s="104"/>
       <c r="AC77" s="14"/>
       <c r="AD77" s="14"/>
-      <c r="AE77" s="117"/>
+      <c r="AE77" s="104"/>
       <c r="AF77" s="14"/>
       <c r="AG77" s="14"/>
       <c r="AH77" s="15"/>
@@ -14995,27 +14995,27 @@
         <f>(($Y$78)*(5*1.08/Misc!$L$18)+0.02*3.75)-0.65</f>
         <v>10.980999999999998</v>
       </c>
-      <c r="AB78" s="117">
+      <c r="AB78" s="104">
         <v>10.7</v>
       </c>
       <c r="AC78" s="14">
-        <f>(($AB$78)*(5*0.92/Misc!$L$19)-0.02*3.75)-0.65</f>
-        <v>9.1190000000000015</v>
+        <f>(($AB$78)*(5*0.92/Misc!$L$19)-0.02*3.75)-0.65-0.05</f>
+        <v>9.0690000000000008</v>
       </c>
       <c r="AD78" s="14">
-        <f>(($AB$78)*(5*1.08/Misc!$L$19)+0.02*3.75)-0.65</f>
-        <v>10.980999999999998</v>
-      </c>
-      <c r="AE78" s="117">
+        <f>(($AB$78)*(5*1.08/Misc!$L$19)+0.02*3.75)-0.65+0.05</f>
+        <v>11.030999999999999</v>
+      </c>
+      <c r="AE78" s="104">
         <v>10.7</v>
       </c>
       <c r="AF78" s="14">
-        <f>(($AE$78)*(5*0.92/Misc!$L$20)-0.02*3.75)-0.65</f>
-        <v>9.1190000000000015</v>
+        <f>(($AE$78)*(5*0.92/Misc!$L$20)-0.02*3.75)-0.65-0.05</f>
+        <v>9.0690000000000008</v>
       </c>
       <c r="AG78" s="14">
-        <f>(($AE$78)*(5*1.08/Misc!$L$20)+0.02*3.75)-0.65</f>
-        <v>10.980999999999998</v>
+        <f>(($AE$78)*(5*1.08/Misc!$L$20)+0.02*3.75)-0.65+0.05</f>
+        <v>11.030999999999999</v>
       </c>
       <c r="AH78" s="15">
         <v>10.7</v>
@@ -15198,27 +15198,27 @@
         <f>(($Y$79)*(5*1.08/Misc!$L$18)+0.02*3.75)-0.65</f>
         <v>11.412999999999998</v>
       </c>
-      <c r="AB79" s="117">
+      <c r="AB79" s="104">
         <v>11.1</v>
       </c>
       <c r="AC79" s="14">
-        <f>(($AB$79)*(5*0.92/Misc!$L$19)-0.02*3.75)-0.65</f>
-        <v>9.4870000000000019</v>
+        <f>(($AB$79)*(5*0.92/Misc!$L$19)-0.02*3.75)-0.65-0.05</f>
+        <v>9.4370000000000012</v>
       </c>
       <c r="AD79" s="14">
-        <f>(($AB$79)*(5*1.08/Misc!$L$19)+0.02*3.75)-0.65</f>
-        <v>11.412999999999998</v>
-      </c>
-      <c r="AE79" s="117">
+        <f>(($AB$79)*(5*1.08/Misc!$L$19)+0.02*3.75)-0.65+0.05</f>
+        <v>11.462999999999999</v>
+      </c>
+      <c r="AE79" s="104">
         <v>11.1</v>
       </c>
       <c r="AF79" s="14">
-        <f>(($AE$79)*(5*0.92/Misc!$L$20)-0.02*3.75)-0.65</f>
-        <v>9.4870000000000019</v>
+        <f>(($AE$79)*(5*0.92/Misc!$L$20)-0.02*3.75)-0.65-0.05</f>
+        <v>9.4370000000000012</v>
       </c>
       <c r="AG79" s="14">
-        <f>(($AE$79)*(5*1.08/Misc!$L$20)+0.02*3.75)-0.65</f>
-        <v>11.412999999999998</v>
+        <f>(($AE$79)*(5*1.08/Misc!$L$20)+0.02*3.75)-0.65+0.05</f>
+        <v>11.462999999999999</v>
       </c>
       <c r="AH79" s="15">
         <v>11.1</v>
@@ -15343,10 +15343,10 @@
       <c r="Y80" s="15"/>
       <c r="Z80" s="14"/>
       <c r="AA80" s="14"/>
-      <c r="AB80" s="117"/>
+      <c r="AB80" s="104"/>
       <c r="AC80" s="14"/>
       <c r="AD80" s="14"/>
-      <c r="AE80" s="117"/>
+      <c r="AE80" s="104"/>
       <c r="AF80" s="14"/>
       <c r="AG80" s="14"/>
       <c r="AH80" s="15"/>
@@ -15466,7 +15466,7 @@
         <f>(Misc!$H$18*5*1.012/Misc!$L$18)+0.02*13.41</f>
         <v>48.844200000000001</v>
       </c>
-      <c r="AB81" s="117">
+      <c r="AB81" s="104">
         <v>48</v>
       </c>
       <c r="AC81" s="14">
@@ -15477,7 +15477,7 @@
         <f>(Misc!$H$19*5*1.012/Misc!$L$19)+0.02*13.41</f>
         <v>48.844200000000001</v>
       </c>
-      <c r="AE81" s="117">
+      <c r="AE81" s="104">
         <v>48</v>
       </c>
       <c r="AF81" s="14">
@@ -15657,7 +15657,7 @@
         <f>(Misc!$I$18*5*1.012/Misc!$L$18)+0.02*13.41</f>
         <v>48.844200000000001</v>
       </c>
-      <c r="AB82" s="117">
+      <c r="AB82" s="104">
         <v>48</v>
       </c>
       <c r="AC82" s="14">
@@ -15668,7 +15668,7 @@
         <f>(Misc!$I$19*5*1.012/Misc!$L$19)+0.02*13.41</f>
         <v>48.844200000000001</v>
       </c>
-      <c r="AE82" s="117">
+      <c r="AE82" s="104">
         <v>48</v>
       </c>
       <c r="AF82" s="14">
@@ -15790,10 +15790,10 @@
       <c r="Y83" s="15"/>
       <c r="Z83" s="14"/>
       <c r="AA83" s="14"/>
-      <c r="AB83" s="117"/>
+      <c r="AB83" s="104"/>
       <c r="AC83" s="14"/>
       <c r="AD83" s="14"/>
-      <c r="AE83" s="117"/>
+      <c r="AE83" s="104"/>
       <c r="AF83" s="14"/>
       <c r="AG83" s="14"/>
       <c r="AH83" s="15"/>
@@ -15913,7 +15913,7 @@
         <f>(Misc!$J$28)*(5*1.008/Misc!$L$18)+0.02*1.1</f>
         <v>5.0317600000000002</v>
       </c>
-      <c r="AB84" s="117">
+      <c r="AB84" s="104">
         <v>4.9960000000000004</v>
       </c>
       <c r="AC84" s="14">
@@ -15924,7 +15924,7 @@
         <f>(Misc!$J$28)*(5*1.008/Misc!$L$19)+0.02*1.1</f>
         <v>5.0317600000000002</v>
       </c>
-      <c r="AE84" s="117">
+      <c r="AE84" s="104">
         <v>4.9960000000000004</v>
       </c>
       <c r="AF84" s="14">
@@ -16104,7 +16104,7 @@
         <f>(Misc!$K$28)*(5*1.008/Misc!$L$18)+0.02*1.1</f>
         <v>5.08216</v>
       </c>
-      <c r="AB85" s="117">
+      <c r="AB85" s="104">
         <v>5</v>
       </c>
       <c r="AC85" s="14">
@@ -16115,7 +16115,7 @@
         <f>(Misc!$K$28)*(5*1.008/Misc!$L$19)+0.02*1.1</f>
         <v>5.08216</v>
       </c>
-      <c r="AE85" s="117">
+      <c r="AE85" s="104">
         <v>5</v>
       </c>
       <c r="AF85" s="14">
@@ -16237,10 +16237,10 @@
       <c r="Y86" s="15"/>
       <c r="Z86" s="14"/>
       <c r="AA86" s="14"/>
-      <c r="AB86" s="117"/>
+      <c r="AB86" s="104"/>
       <c r="AC86" s="14"/>
       <c r="AD86" s="14"/>
-      <c r="AE86" s="117"/>
+      <c r="AE86" s="104"/>
       <c r="AF86" s="14"/>
       <c r="AG86" s="14"/>
       <c r="AH86" s="15"/>
@@ -16360,7 +16360,7 @@
         <f>($Y$87*5*1.072/Misc!$L$18)+0.02*3.4</f>
         <v>2.7480000000000002</v>
       </c>
-      <c r="AB87" s="117">
+      <c r="AB87" s="104">
         <v>2.5</v>
       </c>
       <c r="AC87" s="14">
@@ -16371,7 +16371,7 @@
         <f>($AB$87*5*1.072/Misc!$L$19)+0.02*3.4</f>
         <v>2.7480000000000002</v>
       </c>
-      <c r="AE87" s="117">
+      <c r="AE87" s="104">
         <v>2.5</v>
       </c>
       <c r="AF87" s="14">
@@ -16563,7 +16563,7 @@
         <f>($Y$88*5*1.072/Misc!$L$18)+0.02*3.4</f>
         <v>2.7480000000000002</v>
       </c>
-      <c r="AB88" s="117">
+      <c r="AB88" s="104">
         <v>2.5</v>
       </c>
       <c r="AC88" s="14">
@@ -16574,7 +16574,7 @@
         <f>($AB$88*5*1.072/Misc!$L$19)+0.02*3.4</f>
         <v>2.7480000000000002</v>
       </c>
-      <c r="AE88" s="117">
+      <c r="AE88" s="104">
         <v>2.5</v>
       </c>
       <c r="AF88" s="14">
@@ -16708,10 +16708,10 @@
       <c r="Y89" s="15"/>
       <c r="Z89" s="14"/>
       <c r="AA89" s="14"/>
-      <c r="AB89" s="117"/>
+      <c r="AB89" s="104"/>
       <c r="AC89" s="14"/>
       <c r="AD89" s="14"/>
-      <c r="AE89" s="117"/>
+      <c r="AE89" s="104"/>
       <c r="AF89" s="14"/>
       <c r="AG89" s="14"/>
       <c r="AH89" s="15"/>
@@ -16831,7 +16831,7 @@
         <f>($Y$90*5*1.072/Misc!$L$18)+0.02*3.4</f>
         <v>2.7480000000000002</v>
       </c>
-      <c r="AB90" s="117">
+      <c r="AB90" s="104">
         <v>2.5</v>
       </c>
       <c r="AC90" s="14">
@@ -16842,7 +16842,7 @@
         <f>($AB$90*5*1.072/Misc!$L$19)+0.02*3.4</f>
         <v>2.7480000000000002</v>
       </c>
-      <c r="AE90" s="117">
+      <c r="AE90" s="104">
         <v>2.5</v>
       </c>
       <c r="AF90" s="14">
@@ -17034,7 +17034,7 @@
         <f>($Y$91*5*1.072/Misc!$L$18)+0.02*3.4</f>
         <v>2.7480000000000002</v>
       </c>
-      <c r="AB91" s="117">
+      <c r="AB91" s="104">
         <v>2.5</v>
       </c>
       <c r="AC91" s="14">
@@ -17045,7 +17045,7 @@
         <f>($AB$91*5*1.072/Misc!$L$19)+0.02*3.4</f>
         <v>2.7480000000000002</v>
       </c>
-      <c r="AE91" s="117">
+      <c r="AE91" s="104">
         <v>2.5</v>
       </c>
       <c r="AF91" s="14">
@@ -17179,10 +17179,10 @@
       <c r="Y92" s="15"/>
       <c r="Z92" s="14"/>
       <c r="AA92" s="14"/>
-      <c r="AB92" s="117"/>
+      <c r="AB92" s="104"/>
       <c r="AC92" s="14"/>
       <c r="AD92" s="14"/>
-      <c r="AE92" s="117"/>
+      <c r="AE92" s="104"/>
       <c r="AF92" s="14"/>
       <c r="AG92" s="14"/>
       <c r="AH92" s="15"/>
@@ -17302,27 +17302,27 @@
         <f>($Y$93*5/Misc!$L$18)+0.08</f>
         <v>1.518</v>
       </c>
-      <c r="AB93" s="117">
+      <c r="AB93" s="104">
         <v>1.4379999999999999</v>
       </c>
       <c r="AC93" s="14">
-        <f>($AB$93*5/Misc!$L$19)-0.08</f>
-        <v>1.3579999999999999</v>
+        <f>($AB$93*5/Misc!$L$19)-0.08-0.05</f>
+        <v>1.3079999999999998</v>
       </c>
       <c r="AD93" s="14">
-        <f>($AB$93*5/Misc!$L$19)+0.08</f>
-        <v>1.518</v>
-      </c>
-      <c r="AE93" s="117">
+        <f>($AB$93*5/Misc!$L$19)+0.08+0.05</f>
+        <v>1.5680000000000001</v>
+      </c>
+      <c r="AE93" s="104">
         <v>1.4379999999999999</v>
       </c>
       <c r="AF93" s="14">
-        <f>($AE$93*5/Misc!$L$20)-0.08</f>
-        <v>1.3579999999999999</v>
+        <f>($AE$93*5/Misc!$L$20)-0.08-0.05</f>
+        <v>1.3079999999999998</v>
       </c>
       <c r="AG93" s="14">
-        <f>($AE$93*5/Misc!$L$20)+0.08</f>
-        <v>1.518</v>
+        <f>($AE$93*5/Misc!$L$20)+0.08+0.05</f>
+        <v>1.5680000000000001</v>
       </c>
       <c r="AH93" s="15">
         <v>1.4379999999999999</v>
@@ -17505,27 +17505,27 @@
         <f>($Y$94*5/Misc!$L$18)+0.08</f>
         <v>1.5450000000000002</v>
       </c>
-      <c r="AB94" s="117">
+      <c r="AB94" s="104">
         <v>1.4650000000000001</v>
       </c>
       <c r="AC94" s="14">
-        <f>($AB$94*5/Misc!$L$19)-0.08</f>
-        <v>1.385</v>
+        <f>($AB$94*5/Misc!$L$19)-0.08-0.05</f>
+        <v>1.335</v>
       </c>
       <c r="AD94" s="14">
-        <f>($AB$94*5/Misc!$L$19)+0.08</f>
-        <v>1.5450000000000002</v>
-      </c>
-      <c r="AE94" s="117">
+        <f>($AB$94*5/Misc!$L$19)+0.08+0.05</f>
+        <v>1.5950000000000002</v>
+      </c>
+      <c r="AE94" s="104">
         <v>1.4650000000000001</v>
       </c>
       <c r="AF94" s="14">
-        <f>($AE$94*5/Misc!$L$20)-0.08</f>
-        <v>1.385</v>
+        <f>($AE$94*5/Misc!$L$20)-0.08-0.05</f>
+        <v>1.335</v>
       </c>
       <c r="AG94" s="14">
-        <f>($AE$94*5/Misc!$L$20)+0.08</f>
-        <v>1.5450000000000002</v>
+        <f>($AE$94*5/Misc!$L$20)+0.08+0.05</f>
+        <v>1.5950000000000002</v>
       </c>
       <c r="AH94" s="15">
         <v>1.4650000000000001</v>
@@ -17650,10 +17650,10 @@
       <c r="Y95" s="15"/>
       <c r="Z95" s="14"/>
       <c r="AA95" s="14"/>
-      <c r="AB95" s="117"/>
+      <c r="AB95" s="104"/>
       <c r="AC95" s="14"/>
       <c r="AD95" s="14"/>
-      <c r="AE95" s="117"/>
+      <c r="AE95" s="104"/>
       <c r="AF95" s="14"/>
       <c r="AG95" s="14"/>
       <c r="AH95" s="15"/>
@@ -17731,12 +17731,12 @@
       </c>
       <c r="Z96" s="14"/>
       <c r="AA96" s="14"/>
-      <c r="AB96" s="117">
+      <c r="AB96" s="104">
         <v>160</v>
       </c>
       <c r="AC96" s="14"/>
       <c r="AD96" s="14"/>
-      <c r="AE96" s="117">
+      <c r="AE96" s="104">
         <v>160</v>
       </c>
       <c r="AF96" s="14"/>
@@ -17832,12 +17832,12 @@
       </c>
       <c r="Z97" s="14"/>
       <c r="AA97" s="14"/>
-      <c r="AB97" s="117">
+      <c r="AB97" s="104">
         <v>1</v>
       </c>
       <c r="AC97" s="14"/>
       <c r="AD97" s="14"/>
-      <c r="AE97" s="117">
+      <c r="AE97" s="104">
         <v>1</v>
       </c>
       <c r="AF97" s="14"/>
@@ -17933,12 +17933,12 @@
       </c>
       <c r="Z98" s="14"/>
       <c r="AA98" s="14"/>
-      <c r="AB98" s="117">
+      <c r="AB98" s="104">
         <v>0</v>
       </c>
       <c r="AC98" s="14"/>
       <c r="AD98" s="14"/>
-      <c r="AE98" s="117">
+      <c r="AE98" s="104">
         <v>0</v>
       </c>
       <c r="AF98" s="14"/>
@@ -18034,12 +18034,12 @@
       </c>
       <c r="Z99" s="14"/>
       <c r="AA99" s="14"/>
-      <c r="AB99" s="117">
+      <c r="AB99" s="104">
         <v>1</v>
       </c>
       <c r="AC99" s="14"/>
       <c r="AD99" s="14"/>
-      <c r="AE99" s="117">
+      <c r="AE99" s="104">
         <v>1</v>
       </c>
       <c r="AF99" s="14"/>
@@ -18135,12 +18135,12 @@
       </c>
       <c r="Z100" s="14"/>
       <c r="AA100" s="14"/>
-      <c r="AB100" s="117">
+      <c r="AB100" s="104">
         <v>0</v>
       </c>
       <c r="AC100" s="14"/>
       <c r="AD100" s="14"/>
-      <c r="AE100" s="117">
+      <c r="AE100" s="104">
         <v>0</v>
       </c>
       <c r="AF100" s="14"/>
@@ -18236,12 +18236,12 @@
       </c>
       <c r="Z101" s="14"/>
       <c r="AA101" s="14"/>
-      <c r="AB101" s="117">
+      <c r="AB101" s="104">
         <v>1</v>
       </c>
       <c r="AC101" s="14"/>
       <c r="AD101" s="14"/>
-      <c r="AE101" s="117">
+      <c r="AE101" s="104">
         <v>1</v>
       </c>
       <c r="AF101" s="14"/>
@@ -18337,12 +18337,12 @@
       </c>
       <c r="Z102" s="14"/>
       <c r="AA102" s="14"/>
-      <c r="AB102" s="117">
+      <c r="AB102" s="104">
         <v>0</v>
       </c>
       <c r="AC102" s="14"/>
       <c r="AD102" s="14"/>
-      <c r="AE102" s="117">
+      <c r="AE102" s="104">
         <v>0</v>
       </c>
       <c r="AF102" s="14"/>
@@ -18438,12 +18438,12 @@
       </c>
       <c r="Z103" s="14"/>
       <c r="AA103" s="14"/>
-      <c r="AB103" s="117">
+      <c r="AB103" s="104">
         <v>1</v>
       </c>
       <c r="AC103" s="14"/>
       <c r="AD103" s="14"/>
-      <c r="AE103" s="117">
+      <c r="AE103" s="104">
         <v>1</v>
       </c>
       <c r="AF103" s="14"/>
@@ -18539,12 +18539,12 @@
       </c>
       <c r="Z104" s="14"/>
       <c r="AA104" s="14"/>
-      <c r="AB104" s="117">
+      <c r="AB104" s="104">
         <v>0</v>
       </c>
       <c r="AC104" s="14"/>
       <c r="AD104" s="14"/>
-      <c r="AE104" s="117">
+      <c r="AE104" s="104">
         <v>0</v>
       </c>
       <c r="AF104" s="14"/>
@@ -18640,12 +18640,12 @@
       </c>
       <c r="Z105" s="14"/>
       <c r="AA105" s="14"/>
-      <c r="AB105" s="117">
+      <c r="AB105" s="104">
         <v>1</v>
       </c>
       <c r="AC105" s="14"/>
       <c r="AD105" s="14"/>
-      <c r="AE105" s="117">
+      <c r="AE105" s="104">
         <v>1</v>
       </c>
       <c r="AF105" s="14"/>
@@ -18741,12 +18741,12 @@
       </c>
       <c r="Z106" s="14"/>
       <c r="AA106" s="14"/>
-      <c r="AB106" s="117">
+      <c r="AB106" s="104">
         <v>0</v>
       </c>
       <c r="AC106" s="14"/>
       <c r="AD106" s="14"/>
-      <c r="AE106" s="117">
+      <c r="AE106" s="104">
         <v>0</v>
       </c>
       <c r="AF106" s="14"/>
@@ -18842,12 +18842,12 @@
       </c>
       <c r="Z107" s="14"/>
       <c r="AA107" s="14"/>
-      <c r="AB107" s="117">
+      <c r="AB107" s="104">
         <v>160</v>
       </c>
       <c r="AC107" s="14"/>
       <c r="AD107" s="14"/>
-      <c r="AE107" s="117">
+      <c r="AE107" s="104">
         <v>160</v>
       </c>
       <c r="AF107" s="14"/>
@@ -18985,7 +18985,7 @@
         <f>$Y$108+8</f>
         <v>1008</v>
       </c>
-      <c r="AB108" s="117">
+      <c r="AB108" s="104">
         <v>1000</v>
       </c>
       <c r="AC108" s="14">
@@ -18996,7 +18996,7 @@
         <f>$AB$108+8</f>
         <v>1008</v>
       </c>
-      <c r="AE108" s="117">
+      <c r="AE108" s="104">
         <v>1000</v>
       </c>
       <c r="AF108" s="14">
@@ -19188,7 +19188,7 @@
         <f>$Y$109+8</f>
         <v>1008</v>
       </c>
-      <c r="AB109" s="117">
+      <c r="AB109" s="104">
         <v>1000</v>
       </c>
       <c r="AC109" s="14">
@@ -19199,7 +19199,7 @@
         <f>$AB$109+8</f>
         <v>1008</v>
       </c>
-      <c r="AE109" s="117">
+      <c r="AE109" s="104">
         <v>1000</v>
       </c>
       <c r="AF109" s="14">
@@ -19391,7 +19391,7 @@
         <f>$Y$110+8</f>
         <v>504</v>
       </c>
-      <c r="AB110" s="117">
+      <c r="AB110" s="104">
         <v>496</v>
       </c>
       <c r="AC110" s="14">
@@ -19402,7 +19402,7 @@
         <f>$AB$110+8</f>
         <v>504</v>
       </c>
-      <c r="AE110" s="117">
+      <c r="AE110" s="104">
         <v>496</v>
       </c>
       <c r="AF110" s="14">
@@ -19594,7 +19594,7 @@
         <f>$Y$111+8</f>
         <v>505</v>
       </c>
-      <c r="AB111" s="117">
+      <c r="AB111" s="104">
         <v>497</v>
       </c>
       <c r="AC111" s="14">
@@ -19605,7 +19605,7 @@
         <f>$AB$111+8</f>
         <v>505</v>
       </c>
-      <c r="AE111" s="117">
+      <c r="AE111" s="104">
         <v>497</v>
       </c>
       <c r="AF111" s="14">
@@ -19741,10 +19741,10 @@
       <c r="Y112" s="15"/>
       <c r="Z112" s="14"/>
       <c r="AA112" s="14"/>
-      <c r="AB112" s="117"/>
+      <c r="AB112" s="104"/>
       <c r="AC112" s="14"/>
       <c r="AD112" s="14"/>
-      <c r="AE112" s="117"/>
+      <c r="AE112" s="104"/>
       <c r="AF112" s="14"/>
       <c r="AG112" s="14"/>
       <c r="AH112" s="15"/>
@@ -19822,12 +19822,12 @@
       </c>
       <c r="Z113" s="14"/>
       <c r="AA113" s="14"/>
-      <c r="AB113" s="117">
+      <c r="AB113" s="104">
         <v>160</v>
       </c>
       <c r="AC113" s="14"/>
       <c r="AD113" s="14"/>
-      <c r="AE113" s="117">
+      <c r="AE113" s="104">
         <v>160</v>
       </c>
       <c r="AF113" s="14"/>
@@ -19923,12 +19923,12 @@
       </c>
       <c r="Z114" s="14"/>
       <c r="AA114" s="14"/>
-      <c r="AB114" s="117">
+      <c r="AB114" s="104">
         <v>135</v>
       </c>
       <c r="AC114" s="14"/>
       <c r="AD114" s="14"/>
-      <c r="AE114" s="117">
+      <c r="AE114" s="104">
         <v>135</v>
       </c>
       <c r="AF114" s="14"/>
@@ -20038,14 +20038,14 @@
       <c r="AA115" s="14">
         <v>-81</v>
       </c>
-      <c r="AB115" s="117"/>
+      <c r="AB115" s="104"/>
       <c r="AC115" s="14">
         <v>-206</v>
       </c>
       <c r="AD115" s="14">
         <v>-81</v>
       </c>
-      <c r="AE115" s="117"/>
+      <c r="AE115" s="104"/>
       <c r="AF115" s="14">
         <v>-206</v>
       </c>
@@ -20173,14 +20173,14 @@
       <c r="AA116" s="14">
         <v>1600</v>
       </c>
-      <c r="AB116" s="117"/>
+      <c r="AB116" s="104"/>
       <c r="AC116" s="14">
         <v>-1600</v>
       </c>
       <c r="AD116" s="14">
         <v>1600</v>
       </c>
-      <c r="AE116" s="117"/>
+      <c r="AE116" s="104"/>
       <c r="AF116" s="14">
         <v>-1600</v>
       </c>
@@ -20308,14 +20308,14 @@
       <c r="AA117" s="14">
         <v>207</v>
       </c>
-      <c r="AB117" s="117"/>
+      <c r="AB117" s="104"/>
       <c r="AC117" s="14">
         <v>78</v>
       </c>
       <c r="AD117" s="14">
         <v>207</v>
       </c>
-      <c r="AE117" s="117"/>
+      <c r="AE117" s="104"/>
       <c r="AF117" s="14">
         <v>78</v>
       </c>
@@ -20443,14 +20443,14 @@
       <c r="AA118" s="14">
         <v>1600</v>
       </c>
-      <c r="AB118" s="117"/>
+      <c r="AB118" s="104"/>
       <c r="AC118" s="14">
         <v>-1600</v>
       </c>
       <c r="AD118" s="14">
         <v>1600</v>
       </c>
-      <c r="AE118" s="117"/>
+      <c r="AE118" s="104"/>
       <c r="AF118" s="14">
         <v>-1600</v>
       </c>
@@ -20578,14 +20578,14 @@
       <c r="AA119" s="14">
         <v>-120</v>
       </c>
-      <c r="AB119" s="117"/>
+      <c r="AB119" s="104"/>
       <c r="AC119" s="14">
         <v>-727</v>
       </c>
       <c r="AD119" s="14">
         <v>-120</v>
       </c>
-      <c r="AE119" s="117"/>
+      <c r="AE119" s="104"/>
       <c r="AF119" s="14">
         <v>-727</v>
       </c>
@@ -20713,14 +20713,14 @@
       <c r="AA120" s="14">
         <v>1600</v>
       </c>
-      <c r="AB120" s="117"/>
+      <c r="AB120" s="104"/>
       <c r="AC120" s="14">
         <v>-1600</v>
       </c>
       <c r="AD120" s="14">
         <v>1600</v>
       </c>
-      <c r="AE120" s="117"/>
+      <c r="AE120" s="104"/>
       <c r="AF120" s="14">
         <v>-1600</v>
       </c>
@@ -20876,7 +20876,7 @@
         <f>255*0.001</f>
         <v>0.255</v>
       </c>
-      <c r="AB121" s="117">
+      <c r="AB121" s="104">
         <v>0</v>
       </c>
       <c r="AC121" s="14">
@@ -20887,7 +20887,7 @@
         <f>255*0.001</f>
         <v>0.255</v>
       </c>
-      <c r="AE121" s="117">
+      <c r="AE121" s="104">
         <v>0</v>
       </c>
       <c r="AF121" s="14">
@@ -21079,7 +21079,7 @@
         <f>255*0.001</f>
         <v>0.255</v>
       </c>
-      <c r="AB122" s="117">
+      <c r="AB122" s="104">
         <v>0</v>
       </c>
       <c r="AC122" s="14">
@@ -21090,7 +21090,7 @@
         <f>255*0.001</f>
         <v>0.255</v>
       </c>
-      <c r="AE122" s="117">
+      <c r="AE122" s="104">
         <v>0</v>
       </c>
       <c r="AF122" s="14">
@@ -21282,7 +21282,7 @@
         <f>-395*0.001</f>
         <v>-0.39500000000000002</v>
       </c>
-      <c r="AB123" s="117">
+      <c r="AB123" s="104">
         <v>-1</v>
       </c>
       <c r="AC123" s="14">
@@ -21293,7 +21293,7 @@
         <f>-395*0.001</f>
         <v>-0.39500000000000002</v>
       </c>
-      <c r="AE123" s="117">
+      <c r="AE123" s="104">
         <v>-1</v>
       </c>
       <c r="AF123" s="14">
@@ -21443,12 +21443,12 @@
       </c>
       <c r="Z124" s="14"/>
       <c r="AA124" s="14"/>
-      <c r="AB124" s="117">
+      <c r="AB124" s="104">
         <v>35327</v>
       </c>
       <c r="AC124" s="14"/>
       <c r="AD124" s="14"/>
-      <c r="AE124" s="117">
+      <c r="AE124" s="104">
         <v>35327</v>
       </c>
       <c r="AF124" s="14"/>
@@ -21544,12 +21544,12 @@
       </c>
       <c r="Z125" s="14"/>
       <c r="AA125" s="14"/>
-      <c r="AB125" s="117">
+      <c r="AB125" s="104">
         <v>137</v>
       </c>
       <c r="AC125" s="14"/>
       <c r="AD125" s="14"/>
-      <c r="AE125" s="117">
+      <c r="AE125" s="104">
         <v>137</v>
       </c>
       <c r="AF125" s="14"/>
@@ -21645,12 +21645,12 @@
       </c>
       <c r="Z126" s="14"/>
       <c r="AA126" s="14"/>
-      <c r="AB126" s="117">
+      <c r="AB126" s="104">
         <v>255</v>
       </c>
       <c r="AC126" s="14"/>
       <c r="AD126" s="14"/>
-      <c r="AE126" s="117">
+      <c r="AE126" s="104">
         <v>255</v>
       </c>
       <c r="AF126" s="14"/>
@@ -21746,12 +21746,12 @@
       </c>
       <c r="Z127" s="14"/>
       <c r="AA127" s="14"/>
-      <c r="AB127" s="117">
+      <c r="AB127" s="104">
         <v>4096</v>
       </c>
       <c r="AC127" s="14"/>
       <c r="AD127" s="14"/>
-      <c r="AE127" s="117">
+      <c r="AE127" s="104">
         <v>4096</v>
       </c>
       <c r="AF127" s="14"/>
@@ -21847,12 +21847,12 @@
       </c>
       <c r="Z128" s="14"/>
       <c r="AA128" s="14"/>
-      <c r="AB128" s="117">
+      <c r="AB128" s="104">
         <v>0</v>
       </c>
       <c r="AC128" s="14"/>
       <c r="AD128" s="14"/>
-      <c r="AE128" s="117">
+      <c r="AE128" s="104">
         <v>0</v>
       </c>
       <c r="AF128" s="14"/>
@@ -21948,12 +21948,12 @@
       </c>
       <c r="Z129" s="14"/>
       <c r="AA129" s="14"/>
-      <c r="AB129" s="117">
+      <c r="AB129" s="104">
         <v>0</v>
       </c>
       <c r="AC129" s="14"/>
       <c r="AD129" s="14"/>
-      <c r="AE129" s="117">
+      <c r="AE129" s="104">
         <v>0</v>
       </c>
       <c r="AF129" s="14"/>
@@ -22049,12 +22049,12 @@
       </c>
       <c r="Z130" s="14"/>
       <c r="AA130" s="14"/>
-      <c r="AB130" s="117">
+      <c r="AB130" s="104">
         <v>2</v>
       </c>
       <c r="AC130" s="14"/>
       <c r="AD130" s="14"/>
-      <c r="AE130" s="117">
+      <c r="AE130" s="104">
         <v>2</v>
       </c>
       <c r="AF130" s="14"/>
@@ -22150,12 +22150,12 @@
       </c>
       <c r="Z131" s="14"/>
       <c r="AA131" s="14"/>
-      <c r="AB131" s="117">
+      <c r="AB131" s="104">
         <v>0</v>
       </c>
       <c r="AC131" s="14"/>
       <c r="AD131" s="14"/>
-      <c r="AE131" s="117">
+      <c r="AE131" s="104">
         <v>0</v>
       </c>
       <c r="AF131" s="14"/>
@@ -22251,12 +22251,12 @@
       </c>
       <c r="Z132" s="14"/>
       <c r="AA132" s="14"/>
-      <c r="AB132" s="117">
+      <c r="AB132" s="104">
         <v>0</v>
       </c>
       <c r="AC132" s="14"/>
       <c r="AD132" s="14"/>
-      <c r="AE132" s="117">
+      <c r="AE132" s="104">
         <v>0</v>
       </c>
       <c r="AF132" s="14"/>
@@ -22352,12 +22352,12 @@
       </c>
       <c r="Z133" s="14"/>
       <c r="AA133" s="14"/>
-      <c r="AB133" s="117">
+      <c r="AB133" s="104">
         <v>0</v>
       </c>
       <c r="AC133" s="14"/>
       <c r="AD133" s="14"/>
-      <c r="AE133" s="117">
+      <c r="AE133" s="104">
         <v>0</v>
       </c>
       <c r="AF133" s="14"/>
@@ -22453,12 +22453,12 @@
       </c>
       <c r="Z134" s="14"/>
       <c r="AA134" s="14"/>
-      <c r="AB134" s="117">
+      <c r="AB134" s="104">
         <v>160</v>
       </c>
       <c r="AC134" s="14"/>
       <c r="AD134" s="14"/>
-      <c r="AE134" s="117">
+      <c r="AE134" s="104">
         <v>160</v>
       </c>
       <c r="AF134" s="14"/>
@@ -22554,12 +22554,12 @@
       </c>
       <c r="Z135" s="14"/>
       <c r="AA135" s="14"/>
-      <c r="AB135" s="117">
+      <c r="AB135" s="104">
         <v>1</v>
       </c>
       <c r="AC135" s="14"/>
       <c r="AD135" s="14"/>
-      <c r="AE135" s="117">
+      <c r="AE135" s="104">
         <v>1</v>
       </c>
       <c r="AF135" s="14"/>
@@ -22655,12 +22655,12 @@
       </c>
       <c r="Z136" s="14"/>
       <c r="AA136" s="14"/>
-      <c r="AB136" s="117">
+      <c r="AB136" s="104">
         <v>160</v>
       </c>
       <c r="AC136" s="14"/>
       <c r="AD136" s="14"/>
-      <c r="AE136" s="117">
+      <c r="AE136" s="104">
         <v>160</v>
       </c>
       <c r="AF136" s="14"/>
@@ -22756,12 +22756,12 @@
       </c>
       <c r="Z137" s="14"/>
       <c r="AA137" s="14"/>
-      <c r="AB137" s="117">
+      <c r="AB137" s="104">
         <v>129</v>
       </c>
       <c r="AC137" s="14"/>
       <c r="AD137" s="14"/>
-      <c r="AE137" s="117">
+      <c r="AE137" s="104">
         <v>129</v>
       </c>
       <c r="AF137" s="14"/>
@@ -22857,12 +22857,12 @@
       </c>
       <c r="Z138" s="14"/>
       <c r="AA138" s="14"/>
-      <c r="AB138" s="117">
+      <c r="AB138" s="104">
         <v>1</v>
       </c>
       <c r="AC138" s="14"/>
       <c r="AD138" s="14"/>
-      <c r="AE138" s="117">
+      <c r="AE138" s="104">
         <v>1</v>
       </c>
       <c r="AF138" s="14"/>
@@ -22958,12 +22958,12 @@
       </c>
       <c r="Z139" s="14"/>
       <c r="AA139" s="14"/>
-      <c r="AB139" s="117">
+      <c r="AB139" s="104">
         <v>0</v>
       </c>
       <c r="AC139" s="14"/>
       <c r="AD139" s="14"/>
-      <c r="AE139" s="117">
+      <c r="AE139" s="104">
         <v>0</v>
       </c>
       <c r="AF139" s="14"/>
@@ -23059,12 +23059,12 @@
       </c>
       <c r="Z140" s="14"/>
       <c r="AA140" s="14"/>
-      <c r="AB140" s="117">
+      <c r="AB140" s="104">
         <v>0</v>
       </c>
       <c r="AC140" s="14"/>
       <c r="AD140" s="14"/>
-      <c r="AE140" s="117">
+      <c r="AE140" s="104">
         <v>0</v>
       </c>
       <c r="AF140" s="14"/>
@@ -23160,12 +23160,12 @@
       </c>
       <c r="Z141" s="14"/>
       <c r="AA141" s="14"/>
-      <c r="AB141" s="117">
+      <c r="AB141" s="104">
         <v>0</v>
       </c>
       <c r="AC141" s="14"/>
       <c r="AD141" s="14"/>
-      <c r="AE141" s="117">
+      <c r="AE141" s="104">
         <v>0</v>
       </c>
       <c r="AF141" s="14"/>
@@ -23261,12 +23261,12 @@
       </c>
       <c r="Z142" s="14"/>
       <c r="AA142" s="14"/>
-      <c r="AB142" s="117">
+      <c r="AB142" s="104">
         <v>0</v>
       </c>
       <c r="AC142" s="14"/>
       <c r="AD142" s="14"/>
-      <c r="AE142" s="117">
+      <c r="AE142" s="104">
         <v>0</v>
       </c>
       <c r="AF142" s="14"/>
@@ -23362,12 +23362,12 @@
       </c>
       <c r="Z143" s="14"/>
       <c r="AA143" s="14"/>
-      <c r="AB143" s="117">
+      <c r="AB143" s="104">
         <v>0</v>
       </c>
       <c r="AC143" s="14"/>
       <c r="AD143" s="14"/>
-      <c r="AE143" s="117">
+      <c r="AE143" s="104">
         <v>0</v>
       </c>
       <c r="AF143" s="14"/>
@@ -23463,12 +23463,12 @@
       </c>
       <c r="Z144" s="14"/>
       <c r="AA144" s="14"/>
-      <c r="AB144" s="117">
+      <c r="AB144" s="104">
         <v>0</v>
       </c>
       <c r="AC144" s="14"/>
       <c r="AD144" s="14"/>
-      <c r="AE144" s="117">
+      <c r="AE144" s="104">
         <v>0</v>
       </c>
       <c r="AF144" s="14"/>
@@ -23564,12 +23564,12 @@
       </c>
       <c r="Z145" s="14"/>
       <c r="AA145" s="14"/>
-      <c r="AB145" s="117">
+      <c r="AB145" s="104">
         <v>1</v>
       </c>
       <c r="AC145" s="14"/>
       <c r="AD145" s="14"/>
-      <c r="AE145" s="117">
+      <c r="AE145" s="104">
         <v>1</v>
       </c>
       <c r="AF145" s="14"/>
@@ -23665,12 +23665,12 @@
       </c>
       <c r="Z146" s="14"/>
       <c r="AA146" s="14"/>
-      <c r="AB146" s="117">
+      <c r="AB146" s="104">
         <v>0</v>
       </c>
       <c r="AC146" s="14"/>
       <c r="AD146" s="14"/>
-      <c r="AE146" s="117">
+      <c r="AE146" s="104">
         <v>0</v>
       </c>
       <c r="AF146" s="14"/>
@@ -23766,12 +23766,12 @@
       </c>
       <c r="Z147" s="14"/>
       <c r="AA147" s="14"/>
-      <c r="AB147" s="117">
+      <c r="AB147" s="104">
         <v>0</v>
       </c>
       <c r="AC147" s="14"/>
       <c r="AD147" s="14"/>
-      <c r="AE147" s="117">
+      <c r="AE147" s="104">
         <v>0</v>
       </c>
       <c r="AF147" s="14"/>
@@ -23867,12 +23867,12 @@
       </c>
       <c r="Z148" s="14"/>
       <c r="AA148" s="14"/>
-      <c r="AB148" s="117">
+      <c r="AB148" s="104">
         <v>0</v>
       </c>
       <c r="AC148" s="14"/>
       <c r="AD148" s="14"/>
-      <c r="AE148" s="117">
+      <c r="AE148" s="104">
         <v>0</v>
       </c>
       <c r="AF148" s="14"/>
@@ -23968,12 +23968,12 @@
       </c>
       <c r="Z149" s="14"/>
       <c r="AA149" s="14"/>
-      <c r="AB149" s="117">
+      <c r="AB149" s="104">
         <v>0</v>
       </c>
       <c r="AC149" s="14"/>
       <c r="AD149" s="14"/>
-      <c r="AE149" s="117">
+      <c r="AE149" s="104">
         <v>0</v>
       </c>
       <c r="AF149" s="14"/>
@@ -24069,12 +24069,12 @@
       </c>
       <c r="Z150" s="14"/>
       <c r="AA150" s="14"/>
-      <c r="AB150" s="117">
+      <c r="AB150" s="104">
         <v>0</v>
       </c>
       <c r="AC150" s="14"/>
       <c r="AD150" s="14"/>
-      <c r="AE150" s="117">
+      <c r="AE150" s="104">
         <v>0</v>
       </c>
       <c r="AF150" s="14"/>
@@ -24170,12 +24170,12 @@
       </c>
       <c r="Z151" s="14"/>
       <c r="AA151" s="14"/>
-      <c r="AB151" s="117">
+      <c r="AB151" s="104">
         <v>0</v>
       </c>
       <c r="AC151" s="14"/>
       <c r="AD151" s="14"/>
-      <c r="AE151" s="117">
+      <c r="AE151" s="104">
         <v>0</v>
       </c>
       <c r="AF151" s="14"/>
@@ -24271,12 +24271,12 @@
       </c>
       <c r="Z152" s="14"/>
       <c r="AA152" s="14"/>
-      <c r="AB152" s="117">
+      <c r="AB152" s="104">
         <v>0</v>
       </c>
       <c r="AC152" s="14"/>
       <c r="AD152" s="14"/>
-      <c r="AE152" s="117">
+      <c r="AE152" s="104">
         <v>0</v>
       </c>
       <c r="AF152" s="14"/>
@@ -24372,12 +24372,12 @@
       </c>
       <c r="Z153" s="14"/>
       <c r="AA153" s="14"/>
-      <c r="AB153" s="117">
+      <c r="AB153" s="104">
         <v>0</v>
       </c>
       <c r="AC153" s="14"/>
       <c r="AD153" s="14"/>
-      <c r="AE153" s="117">
+      <c r="AE153" s="104">
         <v>0</v>
       </c>
       <c r="AF153" s="14"/>
@@ -24473,12 +24473,12 @@
       </c>
       <c r="Z154" s="14"/>
       <c r="AA154" s="14"/>
-      <c r="AB154" s="117">
+      <c r="AB154" s="104">
         <v>0</v>
       </c>
       <c r="AC154" s="14"/>
       <c r="AD154" s="14"/>
-      <c r="AE154" s="117">
+      <c r="AE154" s="104">
         <v>0</v>
       </c>
       <c r="AF154" s="14"/>
@@ -24574,12 +24574,12 @@
       </c>
       <c r="Z155" s="14"/>
       <c r="AA155" s="14"/>
-      <c r="AB155" s="117">
+      <c r="AB155" s="104">
         <v>0</v>
       </c>
       <c r="AC155" s="14"/>
       <c r="AD155" s="14"/>
-      <c r="AE155" s="117">
+      <c r="AE155" s="104">
         <v>0</v>
       </c>
       <c r="AF155" s="14"/>
@@ -24675,12 +24675,12 @@
       </c>
       <c r="Z156" s="14"/>
       <c r="AA156" s="14"/>
-      <c r="AB156" s="117">
+      <c r="AB156" s="104">
         <v>0</v>
       </c>
       <c r="AC156" s="14"/>
       <c r="AD156" s="14"/>
-      <c r="AE156" s="117">
+      <c r="AE156" s="104">
         <v>0</v>
       </c>
       <c r="AF156" s="14"/>
@@ -24776,12 +24776,12 @@
       </c>
       <c r="Z157" s="14"/>
       <c r="AA157" s="14"/>
-      <c r="AB157" s="117">
+      <c r="AB157" s="104">
         <v>0</v>
       </c>
       <c r="AC157" s="14"/>
       <c r="AD157" s="14"/>
-      <c r="AE157" s="117">
+      <c r="AE157" s="104">
         <v>0</v>
       </c>
       <c r="AF157" s="14"/>
@@ -24877,12 +24877,12 @@
       </c>
       <c r="Z158" s="14"/>
       <c r="AA158" s="14"/>
-      <c r="AB158" s="117">
+      <c r="AB158" s="104">
         <v>0</v>
       </c>
       <c r="AC158" s="14"/>
       <c r="AD158" s="14"/>
-      <c r="AE158" s="117">
+      <c r="AE158" s="104">
         <v>0</v>
       </c>
       <c r="AF158" s="14"/>
@@ -24978,12 +24978,12 @@
       </c>
       <c r="Z159" s="14"/>
       <c r="AA159" s="14"/>
-      <c r="AB159" s="117">
+      <c r="AB159" s="104">
         <v>0</v>
       </c>
       <c r="AC159" s="14"/>
       <c r="AD159" s="14"/>
-      <c r="AE159" s="117">
+      <c r="AE159" s="104">
         <v>0</v>
       </c>
       <c r="AF159" s="14"/>
@@ -25079,12 +25079,12 @@
       </c>
       <c r="Z160" s="14"/>
       <c r="AA160" s="14"/>
-      <c r="AB160" s="117">
+      <c r="AB160" s="104">
         <v>0</v>
       </c>
       <c r="AC160" s="14"/>
       <c r="AD160" s="14"/>
-      <c r="AE160" s="117">
+      <c r="AE160" s="104">
         <v>0</v>
       </c>
       <c r="AF160" s="14"/>
@@ -25180,12 +25180,12 @@
       </c>
       <c r="Z161" s="14"/>
       <c r="AA161" s="14"/>
-      <c r="AB161" s="117">
+      <c r="AB161" s="104">
         <v>0</v>
       </c>
       <c r="AC161" s="14"/>
       <c r="AD161" s="14"/>
-      <c r="AE161" s="117">
+      <c r="AE161" s="104">
         <v>0</v>
       </c>
       <c r="AF161" s="14"/>
@@ -25281,12 +25281,12 @@
       </c>
       <c r="Z162" s="14"/>
       <c r="AA162" s="14"/>
-      <c r="AB162" s="117">
+      <c r="AB162" s="104">
         <v>0</v>
       </c>
       <c r="AC162" s="14"/>
       <c r="AD162" s="14"/>
-      <c r="AE162" s="117">
+      <c r="AE162" s="104">
         <v>0</v>
       </c>
       <c r="AF162" s="14"/>
@@ -25382,12 +25382,12 @@
       </c>
       <c r="Z163" s="14"/>
       <c r="AA163" s="14"/>
-      <c r="AB163" s="117">
+      <c r="AB163" s="104">
         <v>0</v>
       </c>
       <c r="AC163" s="14"/>
       <c r="AD163" s="14"/>
-      <c r="AE163" s="117">
+      <c r="AE163" s="104">
         <v>0</v>
       </c>
       <c r="AF163" s="14"/>
@@ -25483,12 +25483,12 @@
       </c>
       <c r="Z164" s="14"/>
       <c r="AA164" s="14"/>
-      <c r="AB164" s="117">
+      <c r="AB164" s="104">
         <v>0</v>
       </c>
       <c r="AC164" s="14"/>
       <c r="AD164" s="14"/>
-      <c r="AE164" s="117">
+      <c r="AE164" s="104">
         <v>0</v>
       </c>
       <c r="AF164" s="14"/>
@@ -25584,12 +25584,12 @@
       </c>
       <c r="Z165" s="14"/>
       <c r="AA165" s="14"/>
-      <c r="AB165" s="117">
+      <c r="AB165" s="104">
         <v>0</v>
       </c>
       <c r="AC165" s="14"/>
       <c r="AD165" s="14"/>
-      <c r="AE165" s="117">
+      <c r="AE165" s="104">
         <v>0</v>
       </c>
       <c r="AF165" s="14"/>
@@ -25685,12 +25685,12 @@
       </c>
       <c r="Z166" s="14"/>
       <c r="AA166" s="14"/>
-      <c r="AB166" s="117">
+      <c r="AB166" s="104">
         <v>0</v>
       </c>
       <c r="AC166" s="14"/>
       <c r="AD166" s="14"/>
-      <c r="AE166" s="117">
+      <c r="AE166" s="104">
         <v>0</v>
       </c>
       <c r="AF166" s="14"/>
@@ -25786,12 +25786,12 @@
       </c>
       <c r="Z167" s="14"/>
       <c r="AA167" s="14"/>
-      <c r="AB167" s="117">
+      <c r="AB167" s="104">
         <v>0</v>
       </c>
       <c r="AC167" s="14"/>
       <c r="AD167" s="14"/>
-      <c r="AE167" s="117">
+      <c r="AE167" s="104">
         <v>0</v>
       </c>
       <c r="AF167" s="14"/>
@@ -25887,12 +25887,12 @@
       </c>
       <c r="Z168" s="14"/>
       <c r="AA168" s="14"/>
-      <c r="AB168" s="117">
+      <c r="AB168" s="104">
         <v>0</v>
       </c>
       <c r="AC168" s="14"/>
       <c r="AD168" s="14"/>
-      <c r="AE168" s="117">
+      <c r="AE168" s="104">
         <v>0</v>
       </c>
       <c r="AF168" s="14"/>
@@ -25988,12 +25988,12 @@
       </c>
       <c r="Z169" s="14"/>
       <c r="AA169" s="14"/>
-      <c r="AB169" s="117">
+      <c r="AB169" s="104">
         <v>0</v>
       </c>
       <c r="AC169" s="14"/>
       <c r="AD169" s="14"/>
-      <c r="AE169" s="117">
+      <c r="AE169" s="104">
         <v>0</v>
       </c>
       <c r="AF169" s="14"/>
@@ -26089,12 +26089,12 @@
       </c>
       <c r="Z170" s="14"/>
       <c r="AA170" s="14"/>
-      <c r="AB170" s="117">
+      <c r="AB170" s="104">
         <v>0</v>
       </c>
       <c r="AC170" s="14"/>
       <c r="AD170" s="14"/>
-      <c r="AE170" s="117">
+      <c r="AE170" s="104">
         <v>0</v>
       </c>
       <c r="AF170" s="14"/>
@@ -26190,12 +26190,12 @@
       </c>
       <c r="Z171" s="14"/>
       <c r="AA171" s="14"/>
-      <c r="AB171" s="117">
+      <c r="AB171" s="104">
         <v>0</v>
       </c>
       <c r="AC171" s="14"/>
       <c r="AD171" s="14"/>
-      <c r="AE171" s="117">
+      <c r="AE171" s="104">
         <v>0</v>
       </c>
       <c r="AF171" s="14"/>
@@ -26291,12 +26291,12 @@
       </c>
       <c r="Z172" s="14"/>
       <c r="AA172" s="14"/>
-      <c r="AB172" s="117">
+      <c r="AB172" s="104">
         <v>0</v>
       </c>
       <c r="AC172" s="14"/>
       <c r="AD172" s="14"/>
-      <c r="AE172" s="117">
+      <c r="AE172" s="104">
         <v>0</v>
       </c>
       <c r="AF172" s="14"/>
@@ -26392,12 +26392,12 @@
       </c>
       <c r="Z173" s="14"/>
       <c r="AA173" s="14"/>
-      <c r="AB173" s="117">
+      <c r="AB173" s="104">
         <v>0</v>
       </c>
       <c r="AC173" s="14"/>
       <c r="AD173" s="14"/>
-      <c r="AE173" s="117">
+      <c r="AE173" s="104">
         <v>0</v>
       </c>
       <c r="AF173" s="14"/>
@@ -26493,12 +26493,12 @@
       </c>
       <c r="Z174" s="14"/>
       <c r="AA174" s="14"/>
-      <c r="AB174" s="117">
+      <c r="AB174" s="104">
         <v>0</v>
       </c>
       <c r="AC174" s="14"/>
       <c r="AD174" s="14"/>
-      <c r="AE174" s="117">
+      <c r="AE174" s="104">
         <v>0</v>
       </c>
       <c r="AF174" s="14"/>
@@ -26594,12 +26594,12 @@
       </c>
       <c r="Z175" s="14"/>
       <c r="AA175" s="14"/>
-      <c r="AB175" s="117">
+      <c r="AB175" s="104">
         <v>0</v>
       </c>
       <c r="AC175" s="14"/>
       <c r="AD175" s="14"/>
-      <c r="AE175" s="117">
+      <c r="AE175" s="104">
         <v>0</v>
       </c>
       <c r="AF175" s="14"/>
@@ -26695,12 +26695,12 @@
       </c>
       <c r="Z176" s="14"/>
       <c r="AA176" s="14"/>
-      <c r="AB176" s="117">
+      <c r="AB176" s="104">
         <v>0</v>
       </c>
       <c r="AC176" s="14"/>
       <c r="AD176" s="14"/>
-      <c r="AE176" s="117">
+      <c r="AE176" s="104">
         <v>0</v>
       </c>
       <c r="AF176" s="14"/>
@@ -26796,12 +26796,12 @@
       </c>
       <c r="Z177" s="14"/>
       <c r="AA177" s="14"/>
-      <c r="AB177" s="117">
+      <c r="AB177" s="104">
         <v>0</v>
       </c>
       <c r="AC177" s="14"/>
       <c r="AD177" s="14"/>
-      <c r="AE177" s="117">
+      <c r="AE177" s="104">
         <v>0</v>
       </c>
       <c r="AF177" s="14"/>
@@ -26897,12 +26897,12 @@
       </c>
       <c r="Z178" s="14"/>
       <c r="AA178" s="14"/>
-      <c r="AB178" s="117">
+      <c r="AB178" s="104">
         <v>0</v>
       </c>
       <c r="AC178" s="14"/>
       <c r="AD178" s="14"/>
-      <c r="AE178" s="117">
+      <c r="AE178" s="104">
         <v>0</v>
       </c>
       <c r="AF178" s="14"/>
@@ -26998,12 +26998,12 @@
       </c>
       <c r="Z179" s="14"/>
       <c r="AA179" s="14"/>
-      <c r="AB179" s="117">
+      <c r="AB179" s="104">
         <v>0</v>
       </c>
       <c r="AC179" s="14"/>
       <c r="AD179" s="14"/>
-      <c r="AE179" s="117">
+      <c r="AE179" s="104">
         <v>0</v>
       </c>
       <c r="AF179" s="14"/>
@@ -27099,12 +27099,12 @@
       </c>
       <c r="Z180" s="14"/>
       <c r="AA180" s="14"/>
-      <c r="AB180" s="117">
+      <c r="AB180" s="104">
         <v>0</v>
       </c>
       <c r="AC180" s="14"/>
       <c r="AD180" s="14"/>
-      <c r="AE180" s="117">
+      <c r="AE180" s="104">
         <v>0</v>
       </c>
       <c r="AF180" s="14"/>
@@ -27200,12 +27200,12 @@
       </c>
       <c r="Z181" s="14"/>
       <c r="AA181" s="14"/>
-      <c r="AB181" s="117">
+      <c r="AB181" s="104">
         <v>0</v>
       </c>
       <c r="AC181" s="14"/>
       <c r="AD181" s="14"/>
-      <c r="AE181" s="117">
+      <c r="AE181" s="104">
         <v>0</v>
       </c>
       <c r="AF181" s="14"/>
@@ -27301,12 +27301,12 @@
       </c>
       <c r="Z182" s="14"/>
       <c r="AA182" s="14"/>
-      <c r="AB182" s="117">
+      <c r="AB182" s="104">
         <v>0</v>
       </c>
       <c r="AC182" s="14"/>
       <c r="AD182" s="14"/>
-      <c r="AE182" s="117">
+      <c r="AE182" s="104">
         <v>0</v>
       </c>
       <c r="AF182" s="14"/>
@@ -27402,12 +27402,12 @@
       </c>
       <c r="Z183" s="14"/>
       <c r="AA183" s="14"/>
-      <c r="AB183" s="117">
+      <c r="AB183" s="104">
         <v>0</v>
       </c>
       <c r="AC183" s="14"/>
       <c r="AD183" s="14"/>
-      <c r="AE183" s="117">
+      <c r="AE183" s="104">
         <v>0</v>
       </c>
       <c r="AF183" s="14"/>
@@ -27503,12 +27503,12 @@
       </c>
       <c r="Z184" s="14"/>
       <c r="AA184" s="14"/>
-      <c r="AB184" s="117">
+      <c r="AB184" s="104">
         <v>0</v>
       </c>
       <c r="AC184" s="14"/>
       <c r="AD184" s="14"/>
-      <c r="AE184" s="117">
+      <c r="AE184" s="104">
         <v>0</v>
       </c>
       <c r="AF184" s="14"/>
@@ -27604,12 +27604,12 @@
       </c>
       <c r="Z185" s="14"/>
       <c r="AA185" s="14"/>
-      <c r="AB185" s="117">
+      <c r="AB185" s="104">
         <v>0</v>
       </c>
       <c r="AC185" s="14"/>
       <c r="AD185" s="14"/>
-      <c r="AE185" s="117">
+      <c r="AE185" s="104">
         <v>0</v>
       </c>
       <c r="AF185" s="14"/>
@@ -27705,12 +27705,12 @@
       </c>
       <c r="Z186" s="14"/>
       <c r="AA186" s="14"/>
-      <c r="AB186" s="117">
+      <c r="AB186" s="104">
         <v>0</v>
       </c>
       <c r="AC186" s="14"/>
       <c r="AD186" s="14"/>
-      <c r="AE186" s="117">
+      <c r="AE186" s="104">
         <v>0</v>
       </c>
       <c r="AF186" s="14"/>
@@ -27806,12 +27806,12 @@
       </c>
       <c r="Z187" s="14"/>
       <c r="AA187" s="14"/>
-      <c r="AB187" s="117">
+      <c r="AB187" s="104">
         <v>0</v>
       </c>
       <c r="AC187" s="14"/>
       <c r="AD187" s="14"/>
-      <c r="AE187" s="117">
+      <c r="AE187" s="104">
         <v>0</v>
       </c>
       <c r="AF187" s="14"/>
@@ -27907,12 +27907,12 @@
       </c>
       <c r="Z188" s="14"/>
       <c r="AA188" s="14"/>
-      <c r="AB188" s="117">
+      <c r="AB188" s="104">
         <v>0</v>
       </c>
       <c r="AC188" s="14"/>
       <c r="AD188" s="14"/>
-      <c r="AE188" s="117">
+      <c r="AE188" s="104">
         <v>0</v>
       </c>
       <c r="AF188" s="14"/>
@@ -28008,12 +28008,12 @@
       </c>
       <c r="Z189" s="14"/>
       <c r="AA189" s="14"/>
-      <c r="AB189" s="117">
+      <c r="AB189" s="104">
         <v>0</v>
       </c>
       <c r="AC189" s="14"/>
       <c r="AD189" s="14"/>
-      <c r="AE189" s="117">
+      <c r="AE189" s="104">
         <v>0</v>
       </c>
       <c r="AF189" s="14"/>
@@ -28109,12 +28109,12 @@
       </c>
       <c r="Z190" s="14"/>
       <c r="AA190" s="14"/>
-      <c r="AB190" s="117">
+      <c r="AB190" s="104">
         <v>0</v>
       </c>
       <c r="AC190" s="14"/>
       <c r="AD190" s="14"/>
-      <c r="AE190" s="117">
+      <c r="AE190" s="104">
         <v>0</v>
       </c>
       <c r="AF190" s="14"/>
@@ -28210,12 +28210,12 @@
       </c>
       <c r="Z191" s="14"/>
       <c r="AA191" s="14"/>
-      <c r="AB191" s="117">
+      <c r="AB191" s="104">
         <v>0</v>
       </c>
       <c r="AC191" s="14"/>
       <c r="AD191" s="14"/>
-      <c r="AE191" s="117">
+      <c r="AE191" s="104">
         <v>0</v>
       </c>
       <c r="AF191" s="14"/>
@@ -28311,12 +28311,12 @@
       </c>
       <c r="Z192" s="14"/>
       <c r="AA192" s="14"/>
-      <c r="AB192" s="117">
+      <c r="AB192" s="104">
         <v>0</v>
       </c>
       <c r="AC192" s="14"/>
       <c r="AD192" s="14"/>
-      <c r="AE192" s="117">
+      <c r="AE192" s="104">
         <v>0</v>
       </c>
       <c r="AF192" s="14"/>
@@ -28412,12 +28412,12 @@
       </c>
       <c r="Z193" s="14"/>
       <c r="AA193" s="14"/>
-      <c r="AB193" s="117">
+      <c r="AB193" s="104">
         <v>0</v>
       </c>
       <c r="AC193" s="14"/>
       <c r="AD193" s="14"/>
-      <c r="AE193" s="117">
+      <c r="AE193" s="104">
         <v>0</v>
       </c>
       <c r="AF193" s="14"/>
@@ -28513,12 +28513,12 @@
       </c>
       <c r="Z194" s="14"/>
       <c r="AA194" s="14"/>
-      <c r="AB194" s="117">
+      <c r="AB194" s="104">
         <v>0</v>
       </c>
       <c r="AC194" s="14"/>
       <c r="AD194" s="14"/>
-      <c r="AE194" s="117">
+      <c r="AE194" s="104">
         <v>0</v>
       </c>
       <c r="AF194" s="14"/>
@@ -28614,12 +28614,12 @@
       </c>
       <c r="Z195" s="14"/>
       <c r="AA195" s="14"/>
-      <c r="AB195" s="117">
+      <c r="AB195" s="104">
         <v>0</v>
       </c>
       <c r="AC195" s="14"/>
       <c r="AD195" s="14"/>
-      <c r="AE195" s="117">
+      <c r="AE195" s="104">
         <v>0</v>
       </c>
       <c r="AF195" s="14"/>
@@ -28715,12 +28715,12 @@
       </c>
       <c r="Z196" s="14"/>
       <c r="AA196" s="14"/>
-      <c r="AB196" s="117">
+      <c r="AB196" s="104">
         <v>0</v>
       </c>
       <c r="AC196" s="14"/>
       <c r="AD196" s="14"/>
-      <c r="AE196" s="117">
+      <c r="AE196" s="104">
         <v>0</v>
       </c>
       <c r="AF196" s="14"/>
@@ -28816,12 +28816,12 @@
       </c>
       <c r="Z197" s="14"/>
       <c r="AA197" s="14"/>
-      <c r="AB197" s="117">
+      <c r="AB197" s="104">
         <v>0</v>
       </c>
       <c r="AC197" s="14"/>
       <c r="AD197" s="14"/>
-      <c r="AE197" s="117">
+      <c r="AE197" s="104">
         <v>0</v>
       </c>
       <c r="AF197" s="14"/>
@@ -28917,12 +28917,12 @@
       </c>
       <c r="Z198" s="14"/>
       <c r="AA198" s="14"/>
-      <c r="AB198" s="117">
+      <c r="AB198" s="104">
         <v>0</v>
       </c>
       <c r="AC198" s="14"/>
       <c r="AD198" s="14"/>
-      <c r="AE198" s="117">
+      <c r="AE198" s="104">
         <v>0</v>
       </c>
       <c r="AF198" s="14"/>
@@ -29018,12 +29018,12 @@
       </c>
       <c r="Z199" s="14"/>
       <c r="AA199" s="14"/>
-      <c r="AB199" s="117">
+      <c r="AB199" s="104">
         <v>0</v>
       </c>
       <c r="AC199" s="14"/>
       <c r="AD199" s="14"/>
-      <c r="AE199" s="117">
+      <c r="AE199" s="104">
         <v>0</v>
       </c>
       <c r="AF199" s="14"/>
@@ -29119,12 +29119,12 @@
       </c>
       <c r="Z200" s="14"/>
       <c r="AA200" s="14"/>
-      <c r="AB200" s="117">
+      <c r="AB200" s="104">
         <v>0</v>
       </c>
       <c r="AC200" s="14"/>
       <c r="AD200" s="14"/>
-      <c r="AE200" s="117">
+      <c r="AE200" s="104">
         <v>0</v>
       </c>
       <c r="AF200" s="14"/>
@@ -29220,12 +29220,12 @@
       </c>
       <c r="Z201" s="14"/>
       <c r="AA201" s="14"/>
-      <c r="AB201" s="117">
+      <c r="AB201" s="104">
         <v>0</v>
       </c>
       <c r="AC201" s="14"/>
       <c r="AD201" s="14"/>
-      <c r="AE201" s="117">
+      <c r="AE201" s="104">
         <v>0</v>
       </c>
       <c r="AF201" s="14"/>
@@ -29321,12 +29321,12 @@
       </c>
       <c r="Z202" s="14"/>
       <c r="AA202" s="14"/>
-      <c r="AB202" s="117">
+      <c r="AB202" s="104">
         <v>0</v>
       </c>
       <c r="AC202" s="14"/>
       <c r="AD202" s="14"/>
-      <c r="AE202" s="117">
+      <c r="AE202" s="104">
         <v>0</v>
       </c>
       <c r="AF202" s="14"/>
@@ -29422,12 +29422,12 @@
       </c>
       <c r="Z203" s="14"/>
       <c r="AA203" s="14"/>
-      <c r="AB203" s="117">
+      <c r="AB203" s="104">
         <v>0</v>
       </c>
       <c r="AC203" s="14"/>
       <c r="AD203" s="14"/>
-      <c r="AE203" s="117">
+      <c r="AE203" s="104">
         <v>0</v>
       </c>
       <c r="AF203" s="14"/>
@@ -29523,12 +29523,12 @@
       </c>
       <c r="Z204" s="14"/>
       <c r="AA204" s="14"/>
-      <c r="AB204" s="117">
+      <c r="AB204" s="104">
         <v>0</v>
       </c>
       <c r="AC204" s="14"/>
       <c r="AD204" s="14"/>
-      <c r="AE204" s="117">
+      <c r="AE204" s="104">
         <v>0</v>
       </c>
       <c r="AF204" s="14"/>
@@ -29624,12 +29624,12 @@
       </c>
       <c r="Z205" s="14"/>
       <c r="AA205" s="14"/>
-      <c r="AB205" s="117">
+      <c r="AB205" s="104">
         <v>0</v>
       </c>
       <c r="AC205" s="14"/>
       <c r="AD205" s="14"/>
-      <c r="AE205" s="117">
+      <c r="AE205" s="104">
         <v>0</v>
       </c>
       <c r="AF205" s="14"/>
@@ -29725,12 +29725,12 @@
       </c>
       <c r="Z206" s="14"/>
       <c r="AA206" s="14"/>
-      <c r="AB206" s="117">
+      <c r="AB206" s="104">
         <v>0</v>
       </c>
       <c r="AC206" s="14"/>
       <c r="AD206" s="14"/>
-      <c r="AE206" s="117">
+      <c r="AE206" s="104">
         <v>0</v>
       </c>
       <c r="AF206" s="14"/>
@@ -29826,12 +29826,12 @@
       </c>
       <c r="Z207" s="14"/>
       <c r="AA207" s="14"/>
-      <c r="AB207" s="117">
+      <c r="AB207" s="104">
         <v>0</v>
       </c>
       <c r="AC207" s="14"/>
       <c r="AD207" s="14"/>
-      <c r="AE207" s="117">
+      <c r="AE207" s="104">
         <v>0</v>
       </c>
       <c r="AF207" s="14"/>
@@ -29927,12 +29927,12 @@
       </c>
       <c r="Z208" s="14"/>
       <c r="AA208" s="14"/>
-      <c r="AB208" s="117">
+      <c r="AB208" s="104">
         <v>0</v>
       </c>
       <c r="AC208" s="14"/>
       <c r="AD208" s="14"/>
-      <c r="AE208" s="117">
+      <c r="AE208" s="104">
         <v>0</v>
       </c>
       <c r="AF208" s="14"/>
@@ -30028,12 +30028,12 @@
       </c>
       <c r="Z209" s="14"/>
       <c r="AA209" s="14"/>
-      <c r="AB209" s="117">
+      <c r="AB209" s="104">
         <v>0</v>
       </c>
       <c r="AC209" s="14"/>
       <c r="AD209" s="14"/>
-      <c r="AE209" s="117">
+      <c r="AE209" s="104">
         <v>0</v>
       </c>
       <c r="AF209" s="14"/>
@@ -30129,12 +30129,12 @@
       </c>
       <c r="Z210" s="14"/>
       <c r="AA210" s="14"/>
-      <c r="AB210" s="117">
+      <c r="AB210" s="104">
         <v>0</v>
       </c>
       <c r="AC210" s="14"/>
       <c r="AD210" s="14"/>
-      <c r="AE210" s="117">
+      <c r="AE210" s="104">
         <v>0</v>
       </c>
       <c r="AF210" s="14"/>
@@ -30230,12 +30230,12 @@
       </c>
       <c r="Z211" s="14"/>
       <c r="AA211" s="14"/>
-      <c r="AB211" s="117">
+      <c r="AB211" s="104">
         <v>0</v>
       </c>
       <c r="AC211" s="14"/>
       <c r="AD211" s="14"/>
-      <c r="AE211" s="117">
+      <c r="AE211" s="104">
         <v>0</v>
       </c>
       <c r="AF211" s="14"/>
@@ -30331,12 +30331,12 @@
       </c>
       <c r="Z212" s="14"/>
       <c r="AA212" s="14"/>
-      <c r="AB212" s="117">
+      <c r="AB212" s="104">
         <v>0</v>
       </c>
       <c r="AC212" s="14"/>
       <c r="AD212" s="14"/>
-      <c r="AE212" s="117">
+      <c r="AE212" s="104">
         <v>0</v>
       </c>
       <c r="AF212" s="14"/>
@@ -30432,12 +30432,12 @@
       </c>
       <c r="Z213" s="14"/>
       <c r="AA213" s="14"/>
-      <c r="AB213" s="117">
+      <c r="AB213" s="104">
         <v>0</v>
       </c>
       <c r="AC213" s="14"/>
       <c r="AD213" s="14"/>
-      <c r="AE213" s="117">
+      <c r="AE213" s="104">
         <v>0</v>
       </c>
       <c r="AF213" s="14"/>
@@ -30533,12 +30533,12 @@
       </c>
       <c r="Z214" s="14"/>
       <c r="AA214" s="14"/>
-      <c r="AB214" s="117">
+      <c r="AB214" s="104">
         <v>0</v>
       </c>
       <c r="AC214" s="14"/>
       <c r="AD214" s="14"/>
-      <c r="AE214" s="117">
+      <c r="AE214" s="104">
         <v>0</v>
       </c>
       <c r="AF214" s="14"/>
@@ -30634,12 +30634,12 @@
       </c>
       <c r="Z215" s="14"/>
       <c r="AA215" s="14"/>
-      <c r="AB215" s="117">
+      <c r="AB215" s="104">
         <v>0</v>
       </c>
       <c r="AC215" s="14"/>
       <c r="AD215" s="14"/>
-      <c r="AE215" s="117">
+      <c r="AE215" s="104">
         <v>0</v>
       </c>
       <c r="AF215" s="14"/>
@@ -30735,12 +30735,12 @@
       </c>
       <c r="Z216" s="14"/>
       <c r="AA216" s="14"/>
-      <c r="AB216" s="117">
+      <c r="AB216" s="104">
         <v>0</v>
       </c>
       <c r="AC216" s="14"/>
       <c r="AD216" s="14"/>
-      <c r="AE216" s="117">
+      <c r="AE216" s="104">
         <v>0</v>
       </c>
       <c r="AF216" s="14"/>
@@ -30836,12 +30836,12 @@
       </c>
       <c r="Z217" s="14"/>
       <c r="AA217" s="14"/>
-      <c r="AB217" s="117">
+      <c r="AB217" s="104">
         <v>0</v>
       </c>
       <c r="AC217" s="14"/>
       <c r="AD217" s="14"/>
-      <c r="AE217" s="117">
+      <c r="AE217" s="104">
         <v>0</v>
       </c>
       <c r="AF217" s="14"/>
@@ -30937,12 +30937,12 @@
       </c>
       <c r="Z218" s="14"/>
       <c r="AA218" s="14"/>
-      <c r="AB218" s="117">
+      <c r="AB218" s="104">
         <v>0</v>
       </c>
       <c r="AC218" s="14"/>
       <c r="AD218" s="14"/>
-      <c r="AE218" s="117">
+      <c r="AE218" s="104">
         <v>0</v>
       </c>
       <c r="AF218" s="14"/>
@@ -31038,12 +31038,12 @@
       </c>
       <c r="Z219" s="14"/>
       <c r="AA219" s="14"/>
-      <c r="AB219" s="117">
+      <c r="AB219" s="104">
         <v>0</v>
       </c>
       <c r="AC219" s="14"/>
       <c r="AD219" s="14"/>
-      <c r="AE219" s="117">
+      <c r="AE219" s="104">
         <v>0</v>
       </c>
       <c r="AF219" s="14"/>
@@ -31139,12 +31139,12 @@
       </c>
       <c r="Z220" s="14"/>
       <c r="AA220" s="14"/>
-      <c r="AB220" s="117">
+      <c r="AB220" s="104">
         <v>0</v>
       </c>
       <c r="AC220" s="14"/>
       <c r="AD220" s="14"/>
-      <c r="AE220" s="117">
+      <c r="AE220" s="104">
         <v>0</v>
       </c>
       <c r="AF220" s="14"/>
@@ -31268,7 +31268,7 @@
         <f>Misc!$F$18+3</f>
         <v>4</v>
       </c>
-      <c r="AB221" s="117"/>
+      <c r="AB221" s="104"/>
       <c r="AC221" s="14">
         <f>Misc!$F$19-3</f>
         <v>143</v>
@@ -31277,7 +31277,7 @@
         <f>Misc!$F$19+3</f>
         <v>149</v>
       </c>
-      <c r="AE221" s="117"/>
+      <c r="AE221" s="104"/>
       <c r="AF221" s="14">
         <f>Misc!$F$20-3</f>
         <v>175</v>
@@ -31437,7 +31437,7 @@
         <f>Misc!$G$18+3</f>
         <v>120</v>
       </c>
-      <c r="AB222" s="117"/>
+      <c r="AB222" s="104"/>
       <c r="AC222" s="14">
         <f>Misc!$G$19-3</f>
         <v>143</v>
@@ -31446,7 +31446,7 @@
         <f>Misc!$G$19+3</f>
         <v>149</v>
       </c>
-      <c r="AE222" s="117"/>
+      <c r="AE222" s="104"/>
       <c r="AF222" s="14">
         <f>Misc!$G$20-3</f>
         <v>175</v>
@@ -31606,7 +31606,7 @@
         <f>-(SQRT(2)*Misc!$G$18)+Misc!$O$18</f>
         <v>-153.46298679765212</v>
       </c>
-      <c r="AB223" s="117"/>
+      <c r="AB223" s="104"/>
       <c r="AC223" s="102">
         <f>-(SQRT(2)*Misc!$G$19)-Misc!$O$19</f>
         <v>-218.4751801064719</v>
@@ -31615,7 +31615,7 @@
         <f>-(SQRT(2)*Misc!$G$19)+Misc!$O$19</f>
         <v>-194.4751801064719</v>
       </c>
-      <c r="AE223" s="117"/>
+      <c r="AE223" s="104"/>
       <c r="AF223" s="102">
         <f>-(SQRT(2)*Misc!$F$20)-Misc!$O$20</f>
         <v>-263.73001410241091</v>
@@ -31775,7 +31775,7 @@
         <f>AA223</f>
         <v>-153.46298679765212</v>
       </c>
-      <c r="AB224" s="117"/>
+      <c r="AB224" s="104"/>
       <c r="AC224" s="40">
         <f>AC223</f>
         <v>-218.4751801064719</v>
@@ -31784,7 +31784,7 @@
         <f>AD223</f>
         <v>-194.4751801064719</v>
       </c>
-      <c r="AE224" s="117"/>
+      <c r="AE224" s="104"/>
       <c r="AF224" s="40">
         <f>AF223</f>
         <v>-263.73001410241091</v>
@@ -31944,7 +31944,7 @@
         <f>AA223</f>
         <v>-153.46298679765212</v>
       </c>
-      <c r="AB225" s="117"/>
+      <c r="AB225" s="104"/>
       <c r="AC225" s="40">
         <f>AC223</f>
         <v>-218.4751801064719</v>
@@ -31953,7 +31953,7 @@
         <f>AD223</f>
         <v>-194.4751801064719</v>
       </c>
-      <c r="AE225" s="117"/>
+      <c r="AE225" s="104"/>
       <c r="AF225" s="40">
         <f>AF223</f>
         <v>-263.73001410241091</v>
@@ -32113,7 +32113,7 @@
         <f>-Z223</f>
         <v>177.46298679765212</v>
       </c>
-      <c r="AB226" s="117"/>
+      <c r="AB226" s="104"/>
       <c r="AC226" s="40">
         <f>-AD223</f>
         <v>194.4751801064719</v>
@@ -32122,7 +32122,7 @@
         <f>-AC223</f>
         <v>218.4751801064719</v>
       </c>
-      <c r="AE226" s="117"/>
+      <c r="AE226" s="104"/>
       <c r="AF226" s="40">
         <f>-AG223</f>
         <v>239.73001410241093</v>
@@ -32282,7 +32282,7 @@
         <f t="shared" ref="AA227:AA228" si="11">-Z224</f>
         <v>177.46298679765212</v>
       </c>
-      <c r="AB227" s="117"/>
+      <c r="AB227" s="104"/>
       <c r="AC227" s="40">
         <f t="shared" ref="AC227:AC228" si="12">-AD224</f>
         <v>194.4751801064719</v>
@@ -32291,7 +32291,7 @@
         <f t="shared" ref="AD227:AD228" si="13">-AC224</f>
         <v>218.4751801064719</v>
       </c>
-      <c r="AE227" s="117"/>
+      <c r="AE227" s="104"/>
       <c r="AF227" s="40">
         <f t="shared" ref="AF227:AF228" si="14">-AG224</f>
         <v>239.73001410241093</v>
@@ -32451,7 +32451,7 @@
         <f t="shared" si="11"/>
         <v>177.46298679765212</v>
       </c>
-      <c r="AB228" s="117"/>
+      <c r="AB228" s="104"/>
       <c r="AC228" s="40">
         <f t="shared" si="12"/>
         <v>194.4751801064719</v>
@@ -32460,7 +32460,7 @@
         <f t="shared" si="13"/>
         <v>218.4751801064719</v>
       </c>
-      <c r="AE228" s="117"/>
+      <c r="AE228" s="104"/>
       <c r="AF228" s="40">
         <f t="shared" si="14"/>
         <v>239.73001410241093</v>
@@ -32620,7 +32620,7 @@
         <f>Misc!$N$18</f>
         <v>110</v>
       </c>
-      <c r="AB229" s="117"/>
+      <c r="AB229" s="104"/>
       <c r="AC229" s="14">
         <f>Misc!$M$19</f>
         <v>0</v>
@@ -32629,7 +32629,7 @@
         <f>Misc!$N$19</f>
         <v>110</v>
       </c>
-      <c r="AE229" s="117"/>
+      <c r="AE229" s="104"/>
       <c r="AF229" s="14">
         <f>Misc!$M$20</f>
         <v>0</v>
@@ -32745,10 +32745,10 @@
       <c r="Y230" s="15"/>
       <c r="Z230" s="14"/>
       <c r="AA230" s="14"/>
-      <c r="AB230" s="117"/>
+      <c r="AB230" s="104"/>
       <c r="AC230" s="14"/>
       <c r="AD230" s="14"/>
-      <c r="AE230" s="117"/>
+      <c r="AE230" s="104"/>
       <c r="AF230" s="14"/>
       <c r="AG230" s="14"/>
       <c r="AH230" s="15"/>
@@ -32810,10 +32810,10 @@
       <c r="Y231" s="14"/>
       <c r="Z231" s="14"/>
       <c r="AA231" s="14"/>
-      <c r="AB231" s="117"/>
+      <c r="AB231" s="104"/>
       <c r="AC231" s="14"/>
       <c r="AD231" s="14"/>
-      <c r="AE231" s="117"/>
+      <c r="AE231" s="104"/>
       <c r="AF231" s="14"/>
       <c r="AG231" s="14"/>
       <c r="AH231" s="15"/>
@@ -32875,10 +32875,10 @@
       <c r="Y232" s="14"/>
       <c r="Z232" s="14"/>
       <c r="AA232" s="14"/>
-      <c r="AB232" s="117"/>
+      <c r="AB232" s="104"/>
       <c r="AC232" s="14"/>
       <c r="AD232" s="14"/>
-      <c r="AE232" s="117"/>
+      <c r="AE232" s="104"/>
       <c r="AF232" s="14"/>
       <c r="AG232" s="14"/>
       <c r="AH232" s="15"/>
@@ -33637,16 +33637,16 @@
   <sheetData>
     <row r="3" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="4" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="107" t="s">
+      <c r="B4" s="108" t="s">
         <v>283</v>
       </c>
-      <c r="C4" s="107"/>
-      <c r="E4" s="114" t="s">
+      <c r="C4" s="108"/>
+      <c r="E4" s="115" t="s">
         <v>355</v>
       </c>
-      <c r="F4" s="115"/>
-      <c r="G4" s="115"/>
-      <c r="H4" s="116"/>
+      <c r="F4" s="116"/>
+      <c r="G4" s="116"/>
+      <c r="H4" s="117"/>
       <c r="I4" s="69" t="s">
         <v>284</v>
       </c>
@@ -33723,19 +33723,19 @@
       </c>
     </row>
     <row r="9" spans="2:15" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="E9" s="104" t="s">
+      <c r="E9" s="105" t="s">
         <v>314</v>
       </c>
-      <c r="F9" s="105"/>
-      <c r="G9" s="105"/>
-      <c r="H9" s="105"/>
-      <c r="I9" s="105"/>
-      <c r="J9" s="105"/>
-      <c r="K9" s="105"/>
-      <c r="L9" s="105"/>
-      <c r="M9" s="105"/>
-      <c r="N9" s="105"/>
-      <c r="O9" s="109"/>
+      <c r="F9" s="106"/>
+      <c r="G9" s="106"/>
+      <c r="H9" s="106"/>
+      <c r="I9" s="106"/>
+      <c r="J9" s="106"/>
+      <c r="K9" s="106"/>
+      <c r="L9" s="106"/>
+      <c r="M9" s="106"/>
+      <c r="N9" s="106"/>
+      <c r="O9" s="110"/>
     </row>
     <row r="10" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="E10" s="81" t="s">
@@ -34229,24 +34229,24 @@
     </row>
     <row r="25" spans="5:15" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="26" spans="5:15" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="E26" s="104" t="s">
+      <c r="E26" s="105" t="s">
         <v>325</v>
       </c>
-      <c r="F26" s="108"/>
-      <c r="G26" s="108"/>
-      <c r="H26" s="108"/>
-      <c r="I26" s="108"/>
-      <c r="J26" s="108"/>
-      <c r="K26" s="108"/>
-      <c r="L26" s="108"/>
-      <c r="M26" s="108"/>
-      <c r="N26" s="109"/>
+      <c r="F26" s="109"/>
+      <c r="G26" s="109"/>
+      <c r="H26" s="109"/>
+      <c r="I26" s="109"/>
+      <c r="J26" s="109"/>
+      <c r="K26" s="109"/>
+      <c r="L26" s="109"/>
+      <c r="M26" s="109"/>
+      <c r="N26" s="110"/>
     </row>
     <row r="27" spans="5:15" x14ac:dyDescent="0.3">
-      <c r="E27" s="110" t="s">
+      <c r="E27" s="111" t="s">
         <v>326</v>
       </c>
-      <c r="F27" s="111"/>
+      <c r="F27" s="112"/>
       <c r="G27" s="74" t="s">
         <v>318</v>
       </c>
@@ -34273,8 +34273,8 @@
       </c>
     </row>
     <row r="28" spans="5:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="E28" s="112"/>
-      <c r="F28" s="113"/>
+      <c r="E28" s="113"/>
+      <c r="F28" s="114"/>
       <c r="G28" s="31">
         <v>2.5</v>
       </c>
@@ -34302,19 +34302,19 @@
     </row>
     <row r="30" spans="5:15" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="31" spans="5:15" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="E31" s="104" t="s">
+      <c r="E31" s="105" t="s">
         <v>314</v>
       </c>
-      <c r="F31" s="105"/>
-      <c r="G31" s="105"/>
-      <c r="H31" s="105"/>
-      <c r="I31" s="105"/>
-      <c r="J31" s="105"/>
-      <c r="K31" s="105"/>
-      <c r="L31" s="105"/>
-      <c r="M31" s="105"/>
-      <c r="N31" s="105"/>
-      <c r="O31" s="106"/>
+      <c r="F31" s="106"/>
+      <c r="G31" s="106"/>
+      <c r="H31" s="106"/>
+      <c r="I31" s="106"/>
+      <c r="J31" s="106"/>
+      <c r="K31" s="106"/>
+      <c r="L31" s="106"/>
+      <c r="M31" s="106"/>
+      <c r="N31" s="106"/>
+      <c r="O31" s="107"/>
     </row>
     <row r="32" spans="5:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="E32" s="42" t="s">
@@ -34535,6 +34535,31 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="04cfd3d3-2c89-4764-aaab-c87677d64949">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="50a08be1-ba3e-4a79-8f58-48006bbce96a" xsi:nil="true"/>
+    <_Flow_SignoffStatus xmlns="04cfd3d3-2c89-4764-aaab-c87677d64949" xsi:nil="true"/>
+    <State xmlns="04cfd3d3-2c89-4764-aaab-c87677d64949">New</State>
+    <TaxKeywordTaxHTField xmlns="50a08be1-ba3e-4a79-8f58-48006bbce96a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </TaxKeywordTaxHTField>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101007EAF870E99ECA94F864B327C5B7E3838" ma:contentTypeVersion="31" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="395773d36c2f521a29f182556c34a191">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="04cfd3d3-2c89-4764-aaab-c87677d64949" xmlns:ns3="448318fe-d517-4740-9c4f-0b0645b4226a" xmlns:ns4="50a08be1-ba3e-4a79-8f58-48006bbce96a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fa62a5032f3abd9d41835b1ea6091fec" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="04cfd3d3-2c89-4764-aaab-c87677d64949"/>
@@ -34820,47 +34845,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="04cfd3d3-2c89-4764-aaab-c87677d64949">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="50a08be1-ba3e-4a79-8f58-48006bbce96a" xsi:nil="true"/>
-    <_Flow_SignoffStatus xmlns="04cfd3d3-2c89-4764-aaab-c87677d64949" xsi:nil="true"/>
-    <State xmlns="04cfd3d3-2c89-4764-aaab-c87677d64949">New</State>
-    <TaxKeywordTaxHTField xmlns="50a08be1-ba3e-4a79-8f58-48006bbce96a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </TaxKeywordTaxHTField>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D6E5232F-F37E-427A-A8C4-17F8B14F4745}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1AFA3AA9-6430-449F-9930-F36527A7FEB5}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="04cfd3d3-2c89-4764-aaab-c87677d64949"/>
-    <ds:schemaRef ds:uri="448318fe-d517-4740-9c4f-0b0645b4226a"/>
-    <ds:schemaRef ds:uri="50a08be1-ba3e-4a79-8f58-48006bbce96a"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -34884,15 +34872,27 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1AFA3AA9-6430-449F-9930-F36527A7FEB5}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D6E5232F-F37E-427A-A8C4-17F8B14F4745}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="04cfd3d3-2c89-4764-aaab-c87677d64949"/>
+    <ds:schemaRef ds:uri="448318fe-d517-4740-9c4f-0b0645b4226a"/>
+    <ds:schemaRef ds:uri="50a08be1-ba3e-4a79-8f58-48006bbce96a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
-  <clbl:label id="{3f3ac890-09a1-47d3-8d04-15427d7fec91}" enabled="1" method="Standard" siteId="{39b77101-99b7-41c9-8d6a-7794b9d48476}" contentBits="0" removed="0"/>
+  <clbl:label id="{3f3ac890-09a1-47d3-8d04-15427d7fec91}" enabled="1" method="Standard" siteId="{39b77101-99b7-41c9-8d6a-7794b9d48476}" removed="0"/>
 </clbl:labelList>
 </file>
</xml_diff>